<commit_message>
Recuperados vuelos internacionales en visualizacion ON
</commit_message>
<xml_diff>
--- a/Carga_Real_corto.xlsx
+++ b/Carga_Real_corto.xlsx
@@ -509,9 +509,6 @@
     <t xml:space="preserve">TBC</t>
   </si>
   <si>
-    <t xml:space="preserve">SI</t>
-  </si>
-  <si>
     <t xml:space="preserve">HANSEN-LINDSTROM</t>
   </si>
   <si>
@@ -570,6 +567,9 @@
   </si>
   <si>
     <t xml:space="preserve">Carta Desembarco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SI</t>
   </si>
   <si>
     <t xml:space="preserve">ANNA FRANCINA</t>
@@ -1797,7 +1797,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="105" style="10" width="8.42"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="23.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="23.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -2565,7 +2565,7 @@
     </row>
     <row r="4" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="37" t="s">
-        <v>161</v>
+        <v>106</v>
       </c>
       <c r="B4" s="38" t="s">
         <v>107</v>
@@ -2593,28 +2593,28 @@
         <v>111</v>
       </c>
       <c r="K4" s="40" t="s">
+        <v>161</v>
+      </c>
+      <c r="L4" s="40" t="s">
         <v>162</v>
-      </c>
-      <c r="L4" s="40" t="s">
-        <v>163</v>
       </c>
       <c r="M4" s="37" t="s">
         <v>150</v>
       </c>
       <c r="N4" s="40" t="s">
+        <v>163</v>
+      </c>
+      <c r="O4" s="40" t="s">
         <v>164</v>
       </c>
-      <c r="O4" s="40" t="s">
+      <c r="P4" s="38" t="s">
         <v>165</v>
-      </c>
-      <c r="P4" s="38" t="s">
-        <v>166</v>
       </c>
       <c r="Q4" s="41" t="n">
         <v>21685</v>
       </c>
       <c r="R4" s="40" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="S4" s="40" t="s">
         <v>119</v>
@@ -2626,52 +2626,52 @@
         <v>120</v>
       </c>
       <c r="V4" s="40" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="W4" s="39" t="n">
         <v>45610</v>
       </c>
       <c r="X4" s="39" t="s">
+        <v>168</v>
+      </c>
+      <c r="Y4" s="38" t="s">
         <v>169</v>
-      </c>
-      <c r="Y4" s="38" t="s">
-        <v>170</v>
       </c>
       <c r="Z4" s="39" t="n">
         <v>45610</v>
       </c>
       <c r="AA4" s="39" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB4" s="38" t="s">
         <v>171</v>
-      </c>
-      <c r="AB4" s="38" t="s">
-        <v>172</v>
       </c>
       <c r="AC4" s="39" t="n">
         <v>45611</v>
       </c>
       <c r="AD4" s="39" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AE4" s="38"/>
       <c r="AF4" s="38"/>
       <c r="AG4" s="38"/>
       <c r="AH4" s="40" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AI4" s="39" t="n">
         <v>45611</v>
       </c>
       <c r="AJ4" s="42" t="s">
+        <v>173</v>
+      </c>
+      <c r="AK4" s="45" t="s">
         <v>174</v>
-      </c>
-      <c r="AK4" s="45" t="s">
-        <v>175</v>
       </c>
       <c r="AL4" s="39" t="n">
         <v>45611</v>
       </c>
       <c r="AM4" s="48" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AN4" s="47" t="s">
         <v>130</v>
@@ -2711,10 +2711,10 @@
         <v>45612</v>
       </c>
       <c r="BA4" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="BB4" s="38" t="s">
         <v>177</v>
-      </c>
-      <c r="BB4" s="38" t="s">
-        <v>178</v>
       </c>
       <c r="BC4" s="38"/>
       <c r="BD4" s="39"/>
@@ -18065,7 +18065,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="114" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E1" s="114" t="s">
         <v>4</v>
@@ -18074,13 +18074,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J1" s="14" t="s">
         <v>9</v>
@@ -18340,7 +18340,7 @@
     </row>
     <row r="2" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>161</v>
+        <v>106</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>107</v>
@@ -18361,10 +18361,10 @@
         <v>110</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>161</v>
+        <v>181</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>161</v>
+        <v>181</v>
       </c>
       <c r="K2" s="93" t="s">
         <v>182</v>
@@ -18435,7 +18435,7 @@
         <v>45613</v>
       </c>
       <c r="AY2" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AZ2" s="10" t="s">
         <v>190</v>
@@ -18467,7 +18467,7 @@
     </row>
     <row r="3" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>161</v>
+        <v>106</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>107</v>
@@ -18488,10 +18488,10 @@
         <v>110</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>161</v>
+        <v>181</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>161</v>
+        <v>181</v>
       </c>
       <c r="K3" s="93" t="s">
         <v>191</v>
@@ -18581,7 +18581,7 @@
         <v>45614</v>
       </c>
       <c r="AO3" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AP3" s="10" t="s">
         <v>207</v>
@@ -18596,10 +18596,10 @@
         <v>45615</v>
       </c>
       <c r="AT3" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="AU3" s="10" t="s">
         <v>177</v>
-      </c>
-      <c r="AU3" s="10" t="s">
-        <v>178</v>
       </c>
       <c r="AW3" s="9"/>
       <c r="AX3" s="9"/>

</xml_diff>

<commit_message>
Formateo de excel exportado de visualizacion en proceso. (Faltan tamaños letra, fuente)
</commit_message>
<xml_diff>
--- a/Carga_Real_corto.xlsx
+++ b/Carga_Real_corto.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="215">
   <si>
     <t xml:space="preserve">Activo</t>
   </si>
@@ -32,7 +32,7 @@
     <t xml:space="preserve">Owner</t>
   </si>
   <si>
-    <t xml:space="preserve">Vessel </t>
+    <t xml:space="preserve">Vessel</t>
   </si>
   <si>
     <t xml:space="preserve">Date arrive CL</t>
@@ -65,7 +65,7 @@
     <t xml:space="preserve">Gender</t>
   </si>
   <si>
-    <t xml:space="preserve">Nacionalidad </t>
+    <t xml:space="preserve">Nacionalidad</t>
   </si>
   <si>
     <t xml:space="preserve">Position</t>
@@ -461,6 +461,9 @@
     <t xml:space="preserve">NAVE</t>
   </si>
   <si>
+    <t xml:space="preserve">NORMAL</t>
+  </si>
+  <si>
     <t xml:space="preserve">PUQ Almuerzo</t>
   </si>
   <si>
@@ -560,6 +563,9 @@
     <t xml:space="preserve">Cabo de Hornos</t>
   </si>
   <si>
+    <t xml:space="preserve">Vessel </t>
+  </si>
+  <si>
     <t xml:space="preserve">Date First Flight</t>
   </si>
   <si>
@@ -567,6 +573,9 @@
   </si>
   <si>
     <t xml:space="preserve">Carta Desembarco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nacionalidad </t>
   </si>
   <si>
     <t xml:space="preserve">SI</t>
@@ -672,7 +681,7 @@
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="dd/mm/yy;@"/>
     <numFmt numFmtId="168" formatCode="h:mm"/>
-    <numFmt numFmtId="169" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="169" formatCode="hh:mm:ss"/>
     <numFmt numFmtId="170" formatCode="dd\/mm\/yy"/>
     <numFmt numFmtId="171" formatCode="hh:mm"/>
     <numFmt numFmtId="172" formatCode="hh\/mm\-hh\/mm"/>
@@ -687,7 +696,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -709,7 +717,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -717,33 +724,28 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <strike val="true"/>
@@ -751,27 +753,23 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FFC9211E"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1497,8 +1495,12 @@
   <dxfs count="2">
     <dxf>
       <font>
+        <name val="Calibri"/>
+        <family val="2"/>
         <b val="1"/>
         <i val="0"/>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
       </font>
       <fill>
         <patternFill>
@@ -1508,8 +1510,12 @@
     </dxf>
     <dxf>
       <font>
+        <name val="Calibri"/>
+        <family val="2"/>
         <b val="1"/>
         <i val="0"/>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
       </font>
       <fill>
         <patternFill>
@@ -1726,7 +1732,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="5" width="14.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="13.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="3" width="17.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="5" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="5" width="11.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="6" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="16.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="5" width="17.15"/>
@@ -2117,7 +2123,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="2" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="37" t="s">
         <v>106</v>
       </c>
@@ -2340,9 +2346,11 @@
       <c r="CH2" s="39"/>
       <c r="CI2" s="39"/>
       <c r="CJ2" s="39"/>
-      <c r="CK2" s="38"/>
+      <c r="CK2" s="38" t="s">
+        <v>145</v>
+      </c>
       <c r="CL2" s="38" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="CM2" s="41" t="n">
         <v>42688</v>
@@ -2351,10 +2359,10 @@
         <v>45611</v>
       </c>
       <c r="CO2" s="38" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="CP2" s="38" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CQ2" s="41" t="n">
         <v>45610</v>
@@ -2363,13 +2371,13 @@
         <v>45611</v>
       </c>
       <c r="CS2" s="38" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="CT2" s="38"/>
       <c r="CU2" s="39"/>
       <c r="CV2" s="38"/>
     </row>
-    <row r="3" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
         <v>106</v>
       </c>
@@ -2399,22 +2407,22 @@
         <v>111</v>
       </c>
       <c r="K3" s="40" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L3" s="40" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M3" s="37" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N3" s="40" t="s">
         <v>115</v>
       </c>
       <c r="O3" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P3" s="38" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="Q3" s="41" t="n">
         <v>30432</v>
@@ -2432,22 +2440,22 @@
         <v>120</v>
       </c>
       <c r="V3" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="W3" s="39" t="n">
         <v>45609</v>
       </c>
       <c r="X3" s="39" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="Y3" s="38" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Z3" s="39" t="n">
         <v>45611</v>
       </c>
       <c r="AA3" s="39" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AB3" s="38"/>
       <c r="AC3" s="39"/>
@@ -2456,22 +2464,22 @@
       <c r="AF3" s="38"/>
       <c r="AG3" s="38"/>
       <c r="AH3" s="40" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="AI3" s="39" t="n">
         <v>45611</v>
       </c>
       <c r="AJ3" s="42" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="AK3" s="45" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="AL3" s="39" t="n">
         <v>45611</v>
       </c>
       <c r="AM3" s="46" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="AN3" s="47" t="s">
         <v>130</v>
@@ -2514,7 +2522,7 @@
         <v>138</v>
       </c>
       <c r="BB3" s="38" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="BC3" s="38"/>
       <c r="BD3" s="39"/>
@@ -2563,7 +2571,7 @@
       <c r="CU3" s="39"/>
       <c r="CV3" s="38"/>
     </row>
-    <row r="4" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="37" t="s">
         <v>106</v>
       </c>
@@ -2593,28 +2601,28 @@
         <v>111</v>
       </c>
       <c r="K4" s="40" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L4" s="40" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="M4" s="37" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N4" s="40" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="O4" s="40" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="P4" s="38" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="Q4" s="41" t="n">
         <v>21685</v>
       </c>
       <c r="R4" s="40" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S4" s="40" t="s">
         <v>119</v>
@@ -2626,52 +2634,52 @@
         <v>120</v>
       </c>
       <c r="V4" s="40" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="W4" s="39" t="n">
         <v>45610</v>
       </c>
       <c r="X4" s="39" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="Y4" s="38" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Z4" s="39" t="n">
         <v>45610</v>
       </c>
       <c r="AA4" s="39" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AB4" s="38" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="AC4" s="39" t="n">
         <v>45611</v>
       </c>
       <c r="AD4" s="39" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="AE4" s="38"/>
       <c r="AF4" s="38"/>
       <c r="AG4" s="38"/>
       <c r="AH4" s="40" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="AI4" s="39" t="n">
         <v>45611</v>
       </c>
       <c r="AJ4" s="42" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AK4" s="45" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="AL4" s="39" t="n">
         <v>45611</v>
       </c>
       <c r="AM4" s="48" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AN4" s="47" t="s">
         <v>130</v>
@@ -2711,10 +2719,10 @@
         <v>45612</v>
       </c>
       <c r="BA4" s="38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="BB4" s="38" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="BC4" s="38"/>
       <c r="BD4" s="39"/>
@@ -2799,7 +2807,7 @@
       <c r="CU4" s="39"/>
       <c r="CV4" s="38"/>
     </row>
-    <row r="5" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="37"/>
       <c r="B5" s="38"/>
       <c r="C5" s="38"/>
@@ -2901,7 +2909,7 @@
       <c r="CU5" s="39"/>
       <c r="CV5" s="38"/>
     </row>
-    <row r="6" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="37"/>
       <c r="B6" s="38"/>
       <c r="C6" s="38"/>
@@ -3003,7 +3011,7 @@
       <c r="CU6" s="39"/>
       <c r="CV6" s="38"/>
     </row>
-    <row r="7" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="37"/>
       <c r="B7" s="38"/>
       <c r="C7" s="38"/>
@@ -3105,7 +3113,7 @@
       <c r="CU7" s="39"/>
       <c r="CV7" s="38"/>
     </row>
-    <row r="8" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="37"/>
       <c r="B8" s="38"/>
       <c r="C8" s="38"/>
@@ -3207,7 +3215,7 @@
       <c r="CU8" s="39"/>
       <c r="CV8" s="38"/>
     </row>
-    <row r="9" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="37"/>
       <c r="B9" s="38"/>
       <c r="C9" s="38"/>
@@ -3309,7 +3317,7 @@
       <c r="CU9" s="39"/>
       <c r="CV9" s="38"/>
     </row>
-    <row r="10" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="37"/>
       <c r="B10" s="38"/>
       <c r="C10" s="38"/>
@@ -3411,7 +3419,7 @@
       <c r="CU10" s="39"/>
       <c r="CV10" s="38"/>
     </row>
-    <row r="11" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="37"/>
       <c r="B11" s="38"/>
       <c r="C11" s="38"/>
@@ -3513,7 +3521,7 @@
       <c r="CU11" s="39"/>
       <c r="CV11" s="38"/>
     </row>
-    <row r="12" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="37"/>
       <c r="B12" s="38"/>
       <c r="C12" s="38"/>
@@ -3615,7 +3623,7 @@
       <c r="CU12" s="39"/>
       <c r="CV12" s="38"/>
     </row>
-    <row r="13" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="37"/>
       <c r="B13" s="38"/>
       <c r="C13" s="38"/>
@@ -3717,7 +3725,7 @@
       <c r="CU13" s="39"/>
       <c r="CV13" s="38"/>
     </row>
-    <row r="14" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="37"/>
       <c r="B14" s="38"/>
       <c r="C14" s="38"/>
@@ -3819,7 +3827,7 @@
       <c r="CU14" s="39"/>
       <c r="CV14" s="38"/>
     </row>
-    <row r="15" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="37"/>
       <c r="B15" s="38"/>
       <c r="C15" s="38"/>
@@ -3921,7 +3929,7 @@
       <c r="CU15" s="39"/>
       <c r="CV15" s="38"/>
     </row>
-    <row r="16" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="37"/>
       <c r="B16" s="38"/>
       <c r="C16" s="38"/>
@@ -4023,7 +4031,7 @@
       <c r="CU16" s="39"/>
       <c r="CV16" s="38"/>
     </row>
-    <row r="17" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="37"/>
       <c r="B17" s="38"/>
       <c r="C17" s="38"/>
@@ -4125,7 +4133,7 @@
       <c r="CU17" s="39"/>
       <c r="CV17" s="38"/>
     </row>
-    <row r="18" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="37"/>
       <c r="B18" s="38"/>
       <c r="C18" s="38"/>
@@ -4227,7 +4235,7 @@
       <c r="CU18" s="39"/>
       <c r="CV18" s="38"/>
     </row>
-    <row r="19" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="37"/>
       <c r="B19" s="38"/>
       <c r="C19" s="38"/>
@@ -4329,7 +4337,7 @@
       <c r="CU19" s="39"/>
       <c r="CV19" s="38"/>
     </row>
-    <row r="20" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="37"/>
       <c r="B20" s="38"/>
       <c r="C20" s="38"/>
@@ -4431,7 +4439,7 @@
       <c r="CU20" s="39"/>
       <c r="CV20" s="38"/>
     </row>
-    <row r="21" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="37"/>
       <c r="B21" s="38"/>
       <c r="C21" s="38"/>
@@ -4533,7 +4541,7 @@
       <c r="CU21" s="39"/>
       <c r="CV21" s="38"/>
     </row>
-    <row r="22" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="37"/>
       <c r="B22" s="38"/>
       <c r="C22" s="38"/>
@@ -4635,7 +4643,7 @@
       <c r="CU22" s="39"/>
       <c r="CV22" s="38"/>
     </row>
-    <row r="23" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="37"/>
       <c r="B23" s="38"/>
       <c r="C23" s="38"/>
@@ -4737,7 +4745,7 @@
       <c r="CU23" s="39"/>
       <c r="CV23" s="38"/>
     </row>
-    <row r="24" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="37"/>
       <c r="B24" s="38"/>
       <c r="C24" s="38"/>
@@ -4839,7 +4847,7 @@
       <c r="CU24" s="39"/>
       <c r="CV24" s="38"/>
     </row>
-    <row r="25" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="37"/>
       <c r="B25" s="38"/>
       <c r="C25" s="38"/>
@@ -4941,7 +4949,7 @@
       <c r="CU25" s="39"/>
       <c r="CV25" s="38"/>
     </row>
-    <row r="26" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="37"/>
       <c r="B26" s="38"/>
       <c r="C26" s="38"/>
@@ -5043,7 +5051,7 @@
       <c r="CU26" s="39"/>
       <c r="CV26" s="38"/>
     </row>
-    <row r="27" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="37"/>
       <c r="B27" s="38"/>
       <c r="C27" s="38"/>
@@ -5145,7 +5153,7 @@
       <c r="CU27" s="39"/>
       <c r="CV27" s="38"/>
     </row>
-    <row r="28" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="37"/>
       <c r="B28" s="38"/>
       <c r="C28" s="38"/>
@@ -5247,7 +5255,7 @@
       <c r="CU28" s="39"/>
       <c r="CV28" s="38"/>
     </row>
-    <row r="29" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="37"/>
       <c r="B29" s="38"/>
       <c r="C29" s="38"/>
@@ -5349,7 +5357,7 @@
       <c r="CU29" s="39"/>
       <c r="CV29" s="38"/>
     </row>
-    <row r="30" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="37"/>
       <c r="B30" s="38"/>
       <c r="C30" s="38"/>
@@ -5451,7 +5459,7 @@
       <c r="CU30" s="39"/>
       <c r="CV30" s="38"/>
     </row>
-    <row r="31" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="37"/>
       <c r="B31" s="38"/>
       <c r="C31" s="38"/>
@@ -5553,7 +5561,7 @@
       <c r="CU31" s="39"/>
       <c r="CV31" s="38"/>
     </row>
-    <row r="32" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="37"/>
       <c r="B32" s="38"/>
       <c r="C32" s="38"/>
@@ -5654,7 +5662,7 @@
       <c r="CU32" s="39"/>
       <c r="CV32" s="38"/>
     </row>
-    <row r="33" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="37"/>
       <c r="B33" s="38"/>
       <c r="C33" s="38"/>
@@ -5755,7 +5763,7 @@
       <c r="CU33" s="39"/>
       <c r="CV33" s="38"/>
     </row>
-    <row r="34" s="59" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" s="59" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="50"/>
       <c r="B34" s="51"/>
       <c r="C34" s="51"/>
@@ -5856,7 +5864,7 @@
       <c r="CU34" s="52"/>
       <c r="CV34" s="51"/>
     </row>
-    <row r="35" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="37"/>
       <c r="B35" s="38"/>
       <c r="C35" s="38"/>
@@ -5957,7 +5965,7 @@
       <c r="CU35" s="39"/>
       <c r="CV35" s="38"/>
     </row>
-    <row r="36" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="37"/>
       <c r="B36" s="38"/>
       <c r="C36" s="38"/>
@@ -6064,7 +6072,7 @@
       <c r="DA36" s="39"/>
       <c r="DB36" s="38"/>
     </row>
-    <row r="37" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="37"/>
       <c r="B37" s="38"/>
       <c r="C37" s="38"/>
@@ -6171,7 +6179,7 @@
       <c r="DA37" s="39"/>
       <c r="DB37" s="38"/>
     </row>
-    <row r="38" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="37"/>
       <c r="B38" s="38"/>
       <c r="C38" s="38"/>
@@ -6278,7 +6286,7 @@
       <c r="DA38" s="39"/>
       <c r="DB38" s="38"/>
     </row>
-    <row r="39" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="37"/>
       <c r="B39" s="38"/>
       <c r="C39" s="38"/>
@@ -6385,7 +6393,7 @@
       <c r="DA39" s="39"/>
       <c r="DB39" s="38"/>
     </row>
-    <row r="40" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="37"/>
       <c r="B40" s="38"/>
       <c r="C40" s="38"/>
@@ -6492,7 +6500,7 @@
       <c r="DA40" s="39"/>
       <c r="DB40" s="38"/>
     </row>
-    <row r="41" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="37"/>
       <c r="B41" s="38"/>
       <c r="C41" s="38"/>
@@ -6599,7 +6607,7 @@
       <c r="DA41" s="39"/>
       <c r="DB41" s="38"/>
     </row>
-    <row r="42" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="37"/>
       <c r="B42" s="38"/>
       <c r="C42" s="38"/>
@@ -6701,7 +6709,7 @@
       <c r="CU42" s="39"/>
       <c r="CV42" s="38"/>
     </row>
-    <row r="43" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="37"/>
       <c r="B43" s="38"/>
       <c r="C43" s="38"/>
@@ -6803,7 +6811,7 @@
       <c r="CU43" s="39"/>
       <c r="CV43" s="38"/>
     </row>
-    <row r="44" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="37"/>
       <c r="B44" s="38"/>
       <c r="C44" s="38"/>
@@ -6905,7 +6913,7 @@
       <c r="CU44" s="39"/>
       <c r="CV44" s="38"/>
     </row>
-    <row r="45" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="37"/>
       <c r="B45" s="38"/>
       <c r="C45" s="38"/>
@@ -7007,7 +7015,7 @@
       <c r="CU45" s="39"/>
       <c r="CV45" s="38"/>
     </row>
-    <row r="46" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="37"/>
       <c r="B46" s="38"/>
       <c r="C46" s="38"/>
@@ -7109,7 +7117,7 @@
       <c r="CU46" s="39"/>
       <c r="CV46" s="38"/>
     </row>
-    <row r="47" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="37"/>
       <c r="B47" s="38"/>
       <c r="C47" s="38"/>
@@ -7211,7 +7219,7 @@
       <c r="CU47" s="39"/>
       <c r="CV47" s="38"/>
     </row>
-    <row r="48" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="37"/>
       <c r="B48" s="38"/>
       <c r="C48" s="38"/>
@@ -7313,7 +7321,7 @@
       <c r="CU48" s="39"/>
       <c r="CV48" s="38"/>
     </row>
-    <row r="49" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="37"/>
       <c r="B49" s="38"/>
       <c r="C49" s="38"/>
@@ -7415,7 +7423,7 @@
       <c r="CU49" s="39"/>
       <c r="CV49" s="38"/>
     </row>
-    <row r="50" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="37"/>
       <c r="B50" s="38"/>
       <c r="C50" s="38"/>
@@ -7517,7 +7525,7 @@
       <c r="CU50" s="39"/>
       <c r="CV50" s="38"/>
     </row>
-    <row r="51" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="37"/>
       <c r="B51" s="38"/>
       <c r="C51" s="38"/>
@@ -7619,7 +7627,7 @@
       <c r="CU51" s="39"/>
       <c r="CV51" s="38"/>
     </row>
-    <row r="52" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="37"/>
       <c r="B52" s="38"/>
       <c r="C52" s="38"/>
@@ -7721,7 +7729,7 @@
       <c r="CU52" s="39"/>
       <c r="CV52" s="38"/>
     </row>
-    <row r="53" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="37"/>
       <c r="B53" s="62"/>
       <c r="C53" s="62"/>
@@ -7817,7 +7825,7 @@
       <c r="CU53" s="63"/>
       <c r="CV53" s="62"/>
     </row>
-    <row r="54" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="37"/>
       <c r="B54" s="62"/>
       <c r="C54" s="62"/>
@@ -7913,7 +7921,7 @@
       <c r="CU54" s="63"/>
       <c r="CV54" s="62"/>
     </row>
-    <row r="55" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="37"/>
       <c r="B55" s="62"/>
       <c r="C55" s="62"/>
@@ -8009,7 +8017,7 @@
       <c r="CU55" s="63"/>
       <c r="CV55" s="62"/>
     </row>
-    <row r="56" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="37"/>
       <c r="B56" s="62"/>
       <c r="C56" s="62"/>
@@ -8105,7 +8113,7 @@
       <c r="CU56" s="63"/>
       <c r="CV56" s="62"/>
     </row>
-    <row r="57" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="37"/>
       <c r="B57" s="62"/>
       <c r="C57" s="62"/>
@@ -8201,7 +8209,7 @@
       <c r="CU57" s="63"/>
       <c r="CV57" s="62"/>
     </row>
-    <row r="58" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="62"/>
       <c r="C58" s="62"/>
       <c r="D58" s="63"/>
@@ -8296,7 +8304,7 @@
       <c r="CU58" s="63"/>
       <c r="CV58" s="62"/>
     </row>
-    <row r="59" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="62"/>
       <c r="C59" s="62"/>
       <c r="D59" s="63"/>
@@ -8391,7 +8399,7 @@
       <c r="CU59" s="63"/>
       <c r="CV59" s="62"/>
     </row>
-    <row r="60" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="62"/>
       <c r="C60" s="62"/>
       <c r="D60" s="63"/>
@@ -8486,7 +8494,7 @@
       <c r="CU60" s="63"/>
       <c r="CV60" s="62"/>
     </row>
-    <row r="61" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="62"/>
       <c r="C61" s="62"/>
       <c r="D61" s="63"/>
@@ -8581,7 +8589,7 @@
       <c r="CU61" s="63"/>
       <c r="CV61" s="62"/>
     </row>
-    <row r="62" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="62"/>
       <c r="C62" s="38"/>
       <c r="D62" s="63"/>
@@ -8676,7 +8684,7 @@
       <c r="CU62" s="63"/>
       <c r="CV62" s="62"/>
     </row>
-    <row r="63" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="62"/>
       <c r="C63" s="38"/>
       <c r="D63" s="63"/>
@@ -8771,7 +8779,7 @@
       <c r="CU63" s="63"/>
       <c r="CV63" s="62"/>
     </row>
-    <row r="64" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="62"/>
       <c r="C64" s="38"/>
       <c r="D64" s="63"/>
@@ -8866,7 +8874,7 @@
       <c r="CU64" s="63"/>
       <c r="CV64" s="62"/>
     </row>
-    <row r="65" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="62"/>
       <c r="C65" s="38"/>
       <c r="D65" s="63"/>
@@ -8964,7 +8972,7 @@
       <c r="CU65" s="63"/>
       <c r="CV65" s="62"/>
     </row>
-    <row r="66" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="62"/>
       <c r="C66" s="38"/>
       <c r="D66" s="62"/>
@@ -9061,7 +9069,7 @@
       <c r="CU66" s="63"/>
       <c r="CV66" s="62"/>
     </row>
-    <row r="67" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C67" s="38"/>
       <c r="E67" s="39"/>
       <c r="F67" s="39"/>
@@ -9094,7 +9102,7 @@
       <c r="CQ67" s="41"/>
       <c r="CR67" s="41"/>
     </row>
-    <row r="68" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C68" s="38"/>
       <c r="E68" s="39"/>
       <c r="F68" s="39"/>
@@ -9125,7 +9133,7 @@
       <c r="CC68" s="39"/>
       <c r="CD68" s="42"/>
     </row>
-    <row r="69" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C69" s="38"/>
       <c r="E69" s="39"/>
       <c r="F69" s="39"/>
@@ -9156,7 +9164,7 @@
       <c r="CC69" s="39"/>
       <c r="CD69" s="42"/>
     </row>
-    <row r="70" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E70" s="39"/>
       <c r="F70" s="39"/>
       <c r="I70" s="38"/>
@@ -9185,7 +9193,7 @@
       <c r="CC70" s="39"/>
       <c r="CD70" s="42"/>
     </row>
-    <row r="71" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E71" s="39"/>
       <c r="F71" s="39"/>
       <c r="I71" s="38"/>
@@ -9216,7 +9224,7 @@
       <c r="CC71" s="39"/>
       <c r="CD71" s="42"/>
     </row>
-    <row r="72" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E72" s="39"/>
       <c r="F72" s="39"/>
       <c r="I72" s="38"/>
@@ -9245,7 +9253,7 @@
       <c r="CC72" s="39"/>
       <c r="CD72" s="42"/>
     </row>
-    <row r="73" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C73" s="38"/>
       <c r="E73" s="39"/>
       <c r="F73" s="39"/>
@@ -9277,7 +9285,7 @@
       <c r="CC73" s="39"/>
       <c r="CD73" s="42"/>
     </row>
-    <row r="74" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C74" s="38"/>
       <c r="E74" s="39"/>
       <c r="F74" s="39"/>
@@ -9309,7 +9317,7 @@
       <c r="CC74" s="39"/>
       <c r="CD74" s="42"/>
     </row>
-    <row r="75" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C75" s="38"/>
       <c r="E75" s="39"/>
       <c r="F75" s="39"/>
@@ -9341,7 +9349,7 @@
       <c r="CC75" s="39"/>
       <c r="CD75" s="42"/>
     </row>
-    <row r="76" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C76" s="38"/>
       <c r="E76" s="39"/>
       <c r="F76" s="39"/>
@@ -9373,7 +9381,7 @@
       <c r="CC76" s="39"/>
       <c r="CD76" s="42"/>
     </row>
-    <row r="77" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E77" s="39"/>
       <c r="F77" s="39"/>
       <c r="I77" s="38"/>
@@ -9404,7 +9412,7 @@
       <c r="CC77" s="39"/>
       <c r="CD77" s="42"/>
     </row>
-    <row r="78" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E78" s="39"/>
       <c r="F78" s="39"/>
       <c r="I78" s="38"/>
@@ -9433,7 +9441,7 @@
       <c r="CC78" s="39"/>
       <c r="CD78" s="42"/>
     </row>
-    <row r="79" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E79" s="39"/>
       <c r="F79" s="39"/>
       <c r="I79" s="38"/>
@@ -9462,7 +9470,7 @@
       <c r="CC79" s="39"/>
       <c r="CD79" s="42"/>
     </row>
-    <row r="80" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E80" s="39"/>
       <c r="F80" s="39"/>
       <c r="I80" s="38"/>
@@ -9491,7 +9499,7 @@
       <c r="CC80" s="39"/>
       <c r="CD80" s="42"/>
     </row>
-    <row r="81" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E81" s="39"/>
       <c r="F81" s="39"/>
       <c r="H81" s="72"/>
@@ -9519,7 +9527,7 @@
       <c r="CC81" s="39"/>
       <c r="CD81" s="42"/>
     </row>
-    <row r="82" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E82" s="39"/>
       <c r="F82" s="39"/>
       <c r="H82" s="72"/>
@@ -9547,7 +9555,7 @@
       <c r="CC82" s="39"/>
       <c r="CD82" s="42"/>
     </row>
-    <row r="83" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E83" s="39"/>
       <c r="F83" s="39"/>
       <c r="H83" s="72"/>
@@ -9575,7 +9583,7 @@
       <c r="CC83" s="39"/>
       <c r="CD83" s="42"/>
     </row>
-    <row r="84" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E84" s="39"/>
       <c r="F84" s="39"/>
       <c r="H84" s="72"/>
@@ -9603,7 +9611,7 @@
       <c r="CC84" s="39"/>
       <c r="CD84" s="42"/>
     </row>
-    <row r="85" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E85" s="39"/>
       <c r="F85" s="39"/>
       <c r="H85" s="72"/>
@@ -9631,7 +9639,7 @@
       <c r="CC85" s="39"/>
       <c r="CD85" s="42"/>
     </row>
-    <row r="86" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E86" s="39"/>
       <c r="F86" s="39"/>
       <c r="H86" s="72"/>
@@ -9659,7 +9667,7 @@
       <c r="CC86" s="39"/>
       <c r="CD86" s="42"/>
     </row>
-    <row r="87" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E87" s="39"/>
       <c r="F87" s="39"/>
       <c r="H87" s="72"/>
@@ -9687,7 +9695,7 @@
       <c r="CC87" s="39"/>
       <c r="CD87" s="42"/>
     </row>
-    <row r="88" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E88" s="39"/>
       <c r="F88" s="39"/>
       <c r="H88" s="72"/>
@@ -9715,7 +9723,7 @@
       <c r="CC88" s="39"/>
       <c r="CD88" s="42"/>
     </row>
-    <row r="89" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E89" s="39"/>
       <c r="F89" s="39"/>
       <c r="H89" s="72"/>
@@ -9742,7 +9750,7 @@
       <c r="CC89" s="39"/>
       <c r="CD89" s="42"/>
     </row>
-    <row r="90" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E90" s="39"/>
       <c r="F90" s="39"/>
       <c r="H90" s="72"/>
@@ -9769,7 +9777,7 @@
       <c r="CC90" s="39"/>
       <c r="CD90" s="42"/>
     </row>
-    <row r="91" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E91" s="39"/>
       <c r="F91" s="39"/>
       <c r="H91" s="72"/>
@@ -9796,7 +9804,7 @@
       <c r="CC91" s="39"/>
       <c r="CD91" s="42"/>
     </row>
-    <row r="92" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E92" s="39"/>
       <c r="F92" s="39"/>
       <c r="H92" s="72"/>
@@ -9823,7 +9831,7 @@
       <c r="CC92" s="39"/>
       <c r="CD92" s="42"/>
     </row>
-    <row r="93" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E93" s="39"/>
       <c r="F93" s="39"/>
       <c r="H93" s="72"/>
@@ -9849,7 +9857,7 @@
       <c r="CC93" s="39"/>
       <c r="CD93" s="42"/>
     </row>
-    <row r="94" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E94" s="39"/>
       <c r="F94" s="39"/>
       <c r="H94" s="72"/>
@@ -9875,7 +9883,7 @@
       <c r="CC94" s="39"/>
       <c r="CD94" s="42"/>
     </row>
-    <row r="95" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E95" s="39"/>
       <c r="F95" s="39"/>
       <c r="H95" s="72"/>
@@ -9901,7 +9909,7 @@
       <c r="CC95" s="39"/>
       <c r="CD95" s="42"/>
     </row>
-    <row r="96" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E96" s="39"/>
       <c r="F96" s="39"/>
       <c r="I96" s="38"/>
@@ -9924,7 +9932,7 @@
       <c r="CC96" s="39"/>
       <c r="CD96" s="42"/>
     </row>
-    <row r="97" s="87" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" s="87" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="74"/>
       <c r="B97" s="74"/>
       <c r="C97" s="74"/>
@@ -10026,7 +10034,7 @@
       <c r="CU97" s="86"/>
       <c r="CV97" s="74"/>
     </row>
-    <row r="98" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E98" s="39"/>
       <c r="F98" s="39"/>
       <c r="I98" s="38"/>
@@ -10048,7 +10056,7 @@
       <c r="CC98" s="39"/>
       <c r="CD98" s="42"/>
     </row>
-    <row r="99" s="87" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" s="87" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="74"/>
       <c r="B99" s="74"/>
       <c r="C99" s="74"/>
@@ -10150,7 +10158,7 @@
       <c r="CU99" s="86"/>
       <c r="CV99" s="74"/>
     </row>
-    <row r="100" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E100" s="39"/>
       <c r="F100" s="39"/>
       <c r="I100" s="38"/>
@@ -10174,7 +10182,7 @@
       <c r="CC100" s="39"/>
       <c r="CD100" s="42"/>
     </row>
-    <row r="101" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="37"/>
       <c r="B101" s="37"/>
       <c r="C101" s="37"/>
@@ -10276,7 +10284,7 @@
       <c r="CU101" s="61"/>
       <c r="CV101" s="37"/>
     </row>
-    <row r="102" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="37"/>
       <c r="B102" s="37"/>
       <c r="C102" s="37"/>
@@ -10378,7 +10386,7 @@
       <c r="CU102" s="61"/>
       <c r="CV102" s="37"/>
     </row>
-    <row r="103" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="37"/>
       <c r="B103" s="37"/>
       <c r="C103" s="37"/>
@@ -10480,7 +10488,7 @@
       <c r="CU103" s="61"/>
       <c r="CV103" s="37"/>
     </row>
-    <row r="104" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="37"/>
       <c r="B104" s="37"/>
       <c r="C104" s="37"/>
@@ -10582,7 +10590,7 @@
       <c r="CU104" s="61"/>
       <c r="CV104" s="37"/>
     </row>
-    <row r="105" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="37"/>
       <c r="B105" s="37"/>
       <c r="C105" s="37"/>
@@ -10684,7 +10692,7 @@
       <c r="CU105" s="61"/>
       <c r="CV105" s="37"/>
     </row>
-    <row r="106" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="37"/>
       <c r="B106" s="37"/>
       <c r="C106" s="37"/>
@@ -10786,7 +10794,7 @@
       <c r="CU106" s="61"/>
       <c r="CV106" s="37"/>
     </row>
-    <row r="107" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="37"/>
       <c r="B107" s="37"/>
       <c r="C107" s="37"/>
@@ -10888,7 +10896,7 @@
       <c r="CU107" s="61"/>
       <c r="CV107" s="37"/>
     </row>
-    <row r="108" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="37"/>
       <c r="B108" s="37"/>
       <c r="C108" s="37"/>
@@ -10990,7 +10998,7 @@
       <c r="CU108" s="61"/>
       <c r="CV108" s="37"/>
     </row>
-    <row r="109" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="37"/>
       <c r="B109" s="37"/>
       <c r="C109" s="37"/>
@@ -11092,7 +11100,7 @@
       <c r="CU109" s="61"/>
       <c r="CV109" s="37"/>
     </row>
-    <row r="110" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="37"/>
       <c r="B110" s="37"/>
       <c r="C110" s="37"/>
@@ -11194,7 +11202,7 @@
       <c r="CU110" s="61"/>
       <c r="CV110" s="37"/>
     </row>
-    <row r="111" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="37"/>
       <c r="B111" s="37"/>
       <c r="C111" s="37"/>
@@ -11296,7 +11304,7 @@
       <c r="CU111" s="61"/>
       <c r="CV111" s="37"/>
     </row>
-    <row r="112" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="37"/>
       <c r="B112" s="37"/>
       <c r="C112" s="37"/>
@@ -11398,7 +11406,7 @@
       <c r="CU112" s="61"/>
       <c r="CV112" s="37"/>
     </row>
-    <row r="113" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="37"/>
       <c r="B113" s="37"/>
       <c r="C113" s="37"/>
@@ -11500,7 +11508,7 @@
       <c r="CU113" s="61"/>
       <c r="CV113" s="37"/>
     </row>
-    <row r="114" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="37"/>
       <c r="B114" s="37"/>
       <c r="C114" s="37"/>
@@ -11602,7 +11610,7 @@
       <c r="CU114" s="61"/>
       <c r="CV114" s="37"/>
     </row>
-    <row r="115" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="37"/>
       <c r="B115" s="37"/>
       <c r="C115" s="37"/>
@@ -11704,7 +11712,7 @@
       <c r="CU115" s="61"/>
       <c r="CV115" s="37"/>
     </row>
-    <row r="116" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="37"/>
       <c r="B116" s="37"/>
       <c r="C116" s="37"/>
@@ -11806,7 +11814,7 @@
       <c r="CU116" s="61"/>
       <c r="CV116" s="37"/>
     </row>
-    <row r="117" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="37"/>
       <c r="B117" s="37"/>
       <c r="C117" s="37"/>
@@ -11908,7 +11916,7 @@
       <c r="CU117" s="61"/>
       <c r="CV117" s="37"/>
     </row>
-    <row r="118" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="37"/>
       <c r="B118" s="37"/>
       <c r="C118" s="37"/>
@@ -12010,7 +12018,7 @@
       <c r="CU118" s="61"/>
       <c r="CV118" s="37"/>
     </row>
-    <row r="119" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="37"/>
       <c r="B119" s="37"/>
       <c r="C119" s="37"/>
@@ -12112,7 +12120,7 @@
       <c r="CU119" s="61"/>
       <c r="CV119" s="37"/>
     </row>
-    <row r="120" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="37"/>
       <c r="B120" s="37"/>
       <c r="C120" s="37"/>
@@ -12214,7 +12222,7 @@
       <c r="CU120" s="61"/>
       <c r="CV120" s="37"/>
     </row>
-    <row r="121" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="37"/>
       <c r="B121" s="37"/>
       <c r="C121" s="37"/>
@@ -12316,7 +12324,7 @@
       <c r="CU121" s="61"/>
       <c r="CV121" s="37"/>
     </row>
-    <row r="122" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="37"/>
       <c r="B122" s="37"/>
       <c r="C122" s="37"/>
@@ -12418,7 +12426,7 @@
       <c r="CU122" s="61"/>
       <c r="CV122" s="37"/>
     </row>
-    <row r="123" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="37"/>
       <c r="B123" s="37"/>
       <c r="C123" s="37"/>
@@ -12520,7 +12528,7 @@
       <c r="CU123" s="61"/>
       <c r="CV123" s="37"/>
     </row>
-    <row r="124" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="37"/>
       <c r="B124" s="37"/>
       <c r="C124" s="37"/>
@@ -12622,7 +12630,7 @@
       <c r="CU124" s="61"/>
       <c r="CV124" s="37"/>
     </row>
-    <row r="125" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="37"/>
       <c r="B125" s="37"/>
       <c r="C125" s="37"/>
@@ -12724,7 +12732,7 @@
       <c r="CU125" s="61"/>
       <c r="CV125" s="37"/>
     </row>
-    <row r="126" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="37"/>
       <c r="B126" s="37"/>
       <c r="C126" s="37"/>
@@ -12826,7 +12834,7 @@
       <c r="CU126" s="61"/>
       <c r="CV126" s="37"/>
     </row>
-    <row r="127" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="37"/>
       <c r="B127" s="37"/>
       <c r="C127" s="37"/>
@@ -12928,7 +12936,7 @@
       <c r="CU127" s="61"/>
       <c r="CV127" s="37"/>
     </row>
-    <row r="128" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="37"/>
       <c r="B128" s="37"/>
       <c r="C128" s="37"/>
@@ -13030,7 +13038,7 @@
       <c r="CU128" s="61"/>
       <c r="CV128" s="37"/>
     </row>
-    <row r="129" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="37"/>
       <c r="B129" s="37"/>
       <c r="C129" s="37"/>
@@ -13132,7 +13140,7 @@
       <c r="CU129" s="61"/>
       <c r="CV129" s="37"/>
     </row>
-    <row r="130" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="37"/>
       <c r="B130" s="37"/>
       <c r="C130" s="37"/>
@@ -13234,7 +13242,7 @@
       <c r="CU130" s="61"/>
       <c r="CV130" s="37"/>
     </row>
-    <row r="131" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="37"/>
       <c r="B131" s="37"/>
       <c r="C131" s="37"/>
@@ -13336,7 +13344,7 @@
       <c r="CU131" s="61"/>
       <c r="CV131" s="37"/>
     </row>
-    <row r="132" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="37"/>
       <c r="B132" s="37"/>
       <c r="C132" s="37"/>
@@ -13438,7 +13446,7 @@
       <c r="CU132" s="61"/>
       <c r="CV132" s="37"/>
     </row>
-    <row r="133" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="37"/>
       <c r="B133" s="37"/>
       <c r="C133" s="37"/>
@@ -13540,7 +13548,7 @@
       <c r="CU133" s="61"/>
       <c r="CV133" s="37"/>
     </row>
-    <row r="134" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="37"/>
       <c r="B134" s="37"/>
       <c r="C134" s="37"/>
@@ -13642,7 +13650,7 @@
       <c r="CU134" s="61"/>
       <c r="CV134" s="37"/>
     </row>
-    <row r="135" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="37"/>
       <c r="B135" s="37"/>
       <c r="C135" s="37"/>
@@ -13744,7 +13752,7 @@
       <c r="CU135" s="61"/>
       <c r="CV135" s="37"/>
     </row>
-    <row r="136" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="37"/>
       <c r="B136" s="37"/>
       <c r="C136" s="37"/>
@@ -13846,7 +13854,7 @@
       <c r="CU136" s="61"/>
       <c r="CV136" s="37"/>
     </row>
-    <row r="137" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="37"/>
       <c r="B137" s="37"/>
       <c r="C137" s="37"/>
@@ -13948,7 +13956,7 @@
       <c r="CU137" s="61"/>
       <c r="CV137" s="37"/>
     </row>
-    <row r="138" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="37"/>
       <c r="B138" s="37"/>
       <c r="C138" s="37"/>
@@ -14050,7 +14058,7 @@
       <c r="CU138" s="61"/>
       <c r="CV138" s="37"/>
     </row>
-    <row r="139" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="37"/>
       <c r="B139" s="37"/>
       <c r="C139" s="37"/>
@@ -14152,7 +14160,7 @@
       <c r="CU139" s="61"/>
       <c r="CV139" s="37"/>
     </row>
-    <row r="140" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="37"/>
       <c r="B140" s="37"/>
       <c r="C140" s="37"/>
@@ -14254,7 +14262,7 @@
       <c r="CU140" s="61"/>
       <c r="CV140" s="37"/>
     </row>
-    <row r="141" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="37"/>
       <c r="B141" s="37"/>
       <c r="C141" s="37"/>
@@ -14356,7 +14364,7 @@
       <c r="CU141" s="61"/>
       <c r="CV141" s="37"/>
     </row>
-    <row r="142" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="37"/>
       <c r="B142" s="37"/>
       <c r="C142" s="37"/>
@@ -14458,7 +14466,7 @@
       <c r="CU142" s="61"/>
       <c r="CV142" s="37"/>
     </row>
-    <row r="143" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="37"/>
       <c r="B143" s="37"/>
       <c r="C143" s="37"/>
@@ -14560,7 +14568,7 @@
       <c r="CU143" s="61"/>
       <c r="CV143" s="37"/>
     </row>
-    <row r="144" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="37"/>
       <c r="B144" s="37"/>
       <c r="C144" s="37"/>
@@ -14662,7 +14670,7 @@
       <c r="CU144" s="61"/>
       <c r="CV144" s="37"/>
     </row>
-    <row r="145" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="37"/>
       <c r="B145" s="37"/>
       <c r="C145" s="37"/>
@@ -14764,7 +14772,7 @@
       <c r="CU145" s="61"/>
       <c r="CV145" s="37"/>
     </row>
-    <row r="146" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="37"/>
       <c r="B146" s="37"/>
       <c r="C146" s="37"/>
@@ -14866,7 +14874,7 @@
       <c r="CU146" s="61"/>
       <c r="CV146" s="37"/>
     </row>
-    <row r="147" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="37"/>
       <c r="B147" s="37"/>
       <c r="C147" s="37"/>
@@ -14968,7 +14976,7 @@
       <c r="CU147" s="61"/>
       <c r="CV147" s="37"/>
     </row>
-    <row r="148" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="37"/>
       <c r="B148" s="37"/>
       <c r="C148" s="37"/>
@@ -15070,7 +15078,7 @@
       <c r="CU148" s="61"/>
       <c r="CV148" s="37"/>
     </row>
-    <row r="149" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="37"/>
       <c r="B149" s="37"/>
       <c r="C149" s="37"/>
@@ -15172,7 +15180,7 @@
       <c r="CU149" s="61"/>
       <c r="CV149" s="37"/>
     </row>
-    <row r="150" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="37"/>
       <c r="B150" s="37"/>
       <c r="C150" s="37"/>
@@ -15274,7 +15282,7 @@
       <c r="CU150" s="61"/>
       <c r="CV150" s="37"/>
     </row>
-    <row r="151" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="37"/>
       <c r="B151" s="37"/>
       <c r="C151" s="37"/>
@@ -15376,7 +15384,7 @@
       <c r="CU151" s="61"/>
       <c r="CV151" s="37"/>
     </row>
-    <row r="152" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="37"/>
       <c r="B152" s="37"/>
       <c r="C152" s="37"/>
@@ -15478,7 +15486,7 @@
       <c r="CU152" s="61"/>
       <c r="CV152" s="37"/>
     </row>
-    <row r="153" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="37"/>
       <c r="B153" s="37"/>
       <c r="C153" s="37"/>
@@ -15580,7 +15588,7 @@
       <c r="CU153" s="61"/>
       <c r="CV153" s="37"/>
     </row>
-    <row r="154" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="37"/>
       <c r="B154" s="37"/>
       <c r="C154" s="37"/>
@@ -15682,7 +15690,7 @@
       <c r="CU154" s="61"/>
       <c r="CV154" s="37"/>
     </row>
-    <row r="155" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="37"/>
       <c r="B155" s="37"/>
       <c r="C155" s="37"/>
@@ -15784,7 +15792,7 @@
       <c r="CU155" s="61"/>
       <c r="CV155" s="37"/>
     </row>
-    <row r="156" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E156" s="39"/>
       <c r="F156" s="39"/>
       <c r="I156" s="38"/>
@@ -15813,7 +15821,7 @@
       <c r="CC156" s="39"/>
       <c r="CD156" s="42"/>
     </row>
-    <row r="157" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E157" s="39"/>
       <c r="F157" s="39"/>
       <c r="I157" s="38"/>
@@ -15844,7 +15852,7 @@
       <c r="CD157" s="42"/>
       <c r="CJ157" s="42"/>
     </row>
-    <row r="158" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E158" s="39"/>
       <c r="F158" s="39"/>
       <c r="I158" s="38"/>
@@ -15875,7 +15883,7 @@
       <c r="CD158" s="42"/>
       <c r="CJ158" s="42"/>
     </row>
-    <row r="159" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E159" s="39"/>
       <c r="F159" s="39"/>
       <c r="I159" s="38"/>
@@ -15906,7 +15914,7 @@
       <c r="CD159" s="42"/>
       <c r="CJ159" s="42"/>
     </row>
-    <row r="160" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E160" s="39"/>
       <c r="F160" s="39"/>
       <c r="I160" s="38"/>
@@ -15937,7 +15945,7 @@
       <c r="CD160" s="42"/>
       <c r="CJ160" s="42"/>
     </row>
-    <row r="161" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E161" s="39"/>
       <c r="F161" s="39"/>
       <c r="I161" s="38"/>
@@ -15968,7 +15976,7 @@
       <c r="CD161" s="42"/>
       <c r="CJ161" s="42"/>
     </row>
-    <row r="162" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E162" s="39"/>
       <c r="F162" s="39"/>
       <c r="I162" s="38"/>
@@ -15998,7 +16006,7 @@
       <c r="CD162" s="42"/>
       <c r="CJ162" s="42"/>
     </row>
-    <row r="163" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E163" s="39"/>
       <c r="F163" s="39"/>
       <c r="I163" s="38"/>
@@ -16028,7 +16036,7 @@
       <c r="CD163" s="42"/>
       <c r="CJ163" s="42"/>
     </row>
-    <row r="164" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E164" s="39"/>
       <c r="F164" s="39"/>
       <c r="I164" s="38"/>
@@ -16058,7 +16066,7 @@
       <c r="CD164" s="42"/>
       <c r="CJ164" s="42"/>
     </row>
-    <row r="165" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E165" s="39"/>
       <c r="F165" s="39"/>
       <c r="I165" s="38"/>
@@ -16087,7 +16095,7 @@
       <c r="CD165" s="42"/>
       <c r="CJ165" s="42"/>
     </row>
-    <row r="166" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E166" s="39"/>
       <c r="F166" s="39"/>
       <c r="I166" s="38"/>
@@ -16116,7 +16124,7 @@
       <c r="CD166" s="42"/>
       <c r="CJ166" s="42"/>
     </row>
-    <row r="167" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E167" s="39"/>
       <c r="F167" s="39"/>
       <c r="I167" s="38"/>
@@ -16145,7 +16153,7 @@
       <c r="CD167" s="42"/>
       <c r="CJ167" s="42"/>
     </row>
-    <row r="168" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E168" s="39"/>
       <c r="F168" s="39"/>
       <c r="I168" s="38"/>
@@ -16174,7 +16182,7 @@
       <c r="CD168" s="42"/>
       <c r="CJ168" s="42"/>
     </row>
-    <row r="169" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E169" s="39"/>
       <c r="F169" s="39"/>
       <c r="I169" s="38"/>
@@ -16204,7 +16212,7 @@
       <c r="CD169" s="42"/>
       <c r="CJ169" s="42"/>
     </row>
-    <row r="170" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E170" s="39"/>
       <c r="F170" s="39"/>
       <c r="I170" s="38"/>
@@ -16234,7 +16242,7 @@
       <c r="CD170" s="42"/>
       <c r="CJ170" s="42"/>
     </row>
-    <row r="171" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E171" s="39"/>
       <c r="F171" s="39"/>
       <c r="I171" s="38"/>
@@ -16264,7 +16272,7 @@
       <c r="CD171" s="42"/>
       <c r="CJ171" s="42"/>
     </row>
-    <row r="172" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E172" s="39"/>
       <c r="F172" s="39"/>
       <c r="I172" s="38"/>
@@ -16294,7 +16302,7 @@
       <c r="CD172" s="42"/>
       <c r="CJ172" s="42"/>
     </row>
-    <row r="173" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E173" s="39"/>
       <c r="F173" s="39"/>
       <c r="I173" s="38"/>
@@ -16324,7 +16332,7 @@
       <c r="CD173" s="42"/>
       <c r="CJ173" s="42"/>
     </row>
-    <row r="174" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E174" s="39"/>
       <c r="F174" s="39"/>
       <c r="I174" s="38"/>
@@ -16354,7 +16362,7 @@
       <c r="CD174" s="42"/>
       <c r="CJ174" s="42"/>
     </row>
-    <row r="175" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E175" s="39"/>
       <c r="F175" s="39"/>
       <c r="I175" s="38"/>
@@ -16384,7 +16392,7 @@
       <c r="CD175" s="42"/>
       <c r="CJ175" s="42"/>
     </row>
-    <row r="176" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E176" s="39"/>
       <c r="F176" s="39"/>
       <c r="I176" s="38"/>
@@ -16414,7 +16422,7 @@
       <c r="CD176" s="42"/>
       <c r="CJ176" s="42"/>
     </row>
-    <row r="177" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E177" s="39"/>
       <c r="F177" s="39"/>
       <c r="I177" s="38"/>
@@ -16444,7 +16452,7 @@
       <c r="CD177" s="42"/>
       <c r="CJ177" s="42"/>
     </row>
-    <row r="178" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E178" s="39"/>
       <c r="F178" s="39"/>
       <c r="I178" s="38"/>
@@ -16474,7 +16482,7 @@
       <c r="CD178" s="42"/>
       <c r="CJ178" s="42"/>
     </row>
-    <row r="179" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E179" s="39"/>
       <c r="F179" s="39"/>
       <c r="I179" s="38"/>
@@ -16504,7 +16512,7 @@
       <c r="CD179" s="42"/>
       <c r="CJ179" s="42"/>
     </row>
-    <row r="180" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E180" s="39"/>
       <c r="F180" s="39"/>
       <c r="I180" s="38"/>
@@ -16534,7 +16542,7 @@
       <c r="CD180" s="42"/>
       <c r="CJ180" s="42"/>
     </row>
-    <row r="181" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E181" s="39"/>
       <c r="F181" s="39"/>
       <c r="I181" s="38"/>
@@ -16564,7 +16572,7 @@
       <c r="CD181" s="42"/>
       <c r="CJ181" s="42"/>
     </row>
-    <row r="182" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E182" s="39"/>
       <c r="F182" s="39"/>
       <c r="I182" s="38"/>
@@ -16594,7 +16602,7 @@
       <c r="CD182" s="42"/>
       <c r="CJ182" s="42"/>
     </row>
-    <row r="183" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E183" s="39"/>
       <c r="F183" s="39"/>
       <c r="I183" s="38"/>
@@ -16624,7 +16632,7 @@
       <c r="CD183" s="42"/>
       <c r="CJ183" s="42"/>
     </row>
-    <row r="184" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E184" s="39"/>
       <c r="F184" s="39"/>
       <c r="I184" s="38"/>
@@ -16654,7 +16662,7 @@
       <c r="CD184" s="42"/>
       <c r="CJ184" s="42"/>
     </row>
-    <row r="185" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E185" s="39"/>
       <c r="F185" s="39"/>
       <c r="I185" s="38"/>
@@ -16684,7 +16692,7 @@
       <c r="CD185" s="42"/>
       <c r="CJ185" s="42"/>
     </row>
-    <row r="186" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E186" s="39"/>
       <c r="F186" s="39"/>
       <c r="I186" s="38"/>
@@ -16714,7 +16722,7 @@
       <c r="CD186" s="42"/>
       <c r="CJ186" s="42"/>
     </row>
-    <row r="187" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E187" s="39"/>
       <c r="F187" s="39"/>
       <c r="I187" s="38"/>
@@ -16744,7 +16752,7 @@
       <c r="CD187" s="42"/>
       <c r="CJ187" s="42"/>
     </row>
-    <row r="188" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E188" s="39"/>
       <c r="F188" s="39"/>
       <c r="I188" s="38"/>
@@ -16774,7 +16782,7 @@
       <c r="CD188" s="42"/>
       <c r="CJ188" s="42"/>
     </row>
-    <row r="189" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E189" s="39"/>
       <c r="F189" s="39"/>
       <c r="I189" s="38"/>
@@ -16804,7 +16812,7 @@
       <c r="CD189" s="42"/>
       <c r="CJ189" s="42"/>
     </row>
-    <row r="190" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E190" s="39"/>
       <c r="F190" s="39"/>
       <c r="I190" s="38"/>
@@ -16834,7 +16842,7 @@
       <c r="CD190" s="42"/>
       <c r="CJ190" s="42"/>
     </row>
-    <row r="191" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E191" s="39"/>
       <c r="F191" s="39"/>
       <c r="I191" s="38"/>
@@ -16864,7 +16872,7 @@
       <c r="CD191" s="42"/>
       <c r="CJ191" s="42"/>
     </row>
-    <row r="192" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E192" s="39"/>
       <c r="F192" s="39"/>
       <c r="I192" s="38"/>
@@ -16889,7 +16897,7 @@
       <c r="CD192" s="42"/>
       <c r="CJ192" s="42"/>
     </row>
-    <row r="193" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E193" s="39"/>
       <c r="F193" s="39"/>
       <c r="I193" s="38"/>
@@ -16914,7 +16922,7 @@
       <c r="CD193" s="42"/>
       <c r="CJ193" s="42"/>
     </row>
-    <row r="194" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E194" s="39"/>
       <c r="F194" s="39"/>
       <c r="I194" s="38"/>
@@ -17938,7 +17946,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B2:B50" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B2:B50" type="list">
       <formula1>Clientes</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -18062,10 +18070,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>2</v>
+        <v>179</v>
       </c>
       <c r="D1" s="114" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E1" s="114" t="s">
         <v>4</v>
@@ -18074,13 +18082,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="J1" s="14" t="s">
         <v>9</v>
@@ -18095,7 +18103,7 @@
         <v>12</v>
       </c>
       <c r="N1" s="31" t="s">
-        <v>13</v>
+        <v>183</v>
       </c>
       <c r="O1" s="31" t="s">
         <v>14</v>
@@ -18361,28 +18369,28 @@
         <v>110</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="K2" s="93" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="M2" s="37" t="s">
         <v>114</v>
       </c>
       <c r="N2" s="44" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="O2" s="44" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="P2" s="93" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="Q2" s="61" t="n">
         <v>26176</v>
@@ -18400,13 +18408,13 @@
         <v>120</v>
       </c>
       <c r="V2" s="44" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="W2" s="5"/>
       <c r="Z2" s="9"/>
       <c r="AA2" s="123"/>
       <c r="AB2" s="124" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AC2" s="9" t="n">
         <v>45613</v>
@@ -18426,7 +18434,7 @@
       <c r="AR2" s="5"/>
       <c r="AS2" s="5"/>
       <c r="AV2" s="10" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AW2" s="5" t="n">
         <v>45612</v>
@@ -18435,10 +18443,10 @@
         <v>45613</v>
       </c>
       <c r="AY2" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AZ2" s="10" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="BA2" s="62"/>
       <c r="BB2" s="62"/>
@@ -18488,61 +18496,61 @@
         <v>110</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="K3" s="93" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="M3" s="37" t="s">
         <v>114</v>
       </c>
       <c r="N3" s="44" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="O3" s="44" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="P3" s="93" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="Q3" s="61" t="n">
         <v>34604</v>
       </c>
       <c r="R3" s="44" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="S3" s="44" t="s">
         <v>119</v>
       </c>
       <c r="T3" s="44" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="V3" s="44" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="W3" s="9" t="n">
         <v>45614</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="Y3" s="93" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Z3" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="AA3" s="123" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AB3" s="124" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="AC3" s="9" t="n">
         <v>45615</v>
@@ -18554,25 +18562,25 @@
         <v>132</v>
       </c>
       <c r="AF3" s="64" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="AG3" s="38" t="s">
         <v>134</v>
       </c>
       <c r="AH3" s="64" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="AI3" s="38" t="s">
         <v>134</v>
       </c>
       <c r="AJ3" s="10" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="AK3" s="92" t="n">
         <v>1</v>
       </c>
       <c r="AL3" s="62" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="AM3" s="9" t="n">
         <v>45612</v>
@@ -18581,10 +18589,10 @@
         <v>45614</v>
       </c>
       <c r="AO3" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AP3" s="10" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="AQ3" s="10" t="s">
         <v>137</v>
@@ -18596,10 +18604,10 @@
         <v>45615</v>
       </c>
       <c r="AT3" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AU3" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AW3" s="9"/>
       <c r="AX3" s="9"/>
@@ -18674,10 +18682,10 @@
         <v>0.0701388888888889</v>
       </c>
       <c r="BY3" s="1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="BZ3" s="10" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="CA3" s="113" t="n">
         <v>45612</v>
@@ -18686,10 +18694,10 @@
         <v>45613</v>
       </c>
       <c r="CC3" s="10" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="CD3" s="10" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="CE3" s="113" t="n">
         <v>45612</v>
@@ -18698,7 +18706,7 @@
         <v>45613</v>
       </c>
       <c r="CG3" s="10" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22530,7 +22538,7 @@
       <c r="AH84" s="64"/>
       <c r="BP84" s="10"/>
     </row>
-    <row r="85" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H85" s="37"/>
       <c r="K85" s="3"/>
       <c r="L85" s="3"/>
@@ -22544,7 +22552,7 @@
       <c r="AG85" s="38"/>
       <c r="AH85" s="64"/>
     </row>
-    <row r="86" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H86" s="37"/>
       <c r="K86" s="3"/>
       <c r="L86" s="3"/>
@@ -22558,7 +22566,7 @@
       <c r="AG86" s="38"/>
       <c r="AH86" s="64"/>
     </row>
-    <row r="87" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H87" s="37"/>
       <c r="K87" s="3"/>
       <c r="L87" s="3"/>
@@ -22572,7 +22580,7 @@
       <c r="AG87" s="38"/>
       <c r="AH87" s="64"/>
     </row>
-    <row r="88" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H88" s="37"/>
       <c r="K88" s="3"/>
       <c r="L88" s="3"/>
@@ -22586,7 +22594,7 @@
       <c r="AG88" s="38"/>
       <c r="AH88" s="64"/>
     </row>
-    <row r="89" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H89" s="37"/>
       <c r="K89" s="3"/>
       <c r="L89" s="3"/>
@@ -22600,7 +22608,7 @@
       <c r="AG89" s="38"/>
       <c r="AH89" s="64"/>
     </row>
-    <row r="90" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H90" s="37"/>
       <c r="K90" s="3"/>
       <c r="L90" s="3"/>
@@ -22614,7 +22622,7 @@
       <c r="AG90" s="38"/>
       <c r="AH90" s="64"/>
     </row>
-    <row r="91" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H91" s="37"/>
       <c r="K91" s="3"/>
       <c r="L91" s="3"/>
@@ -22628,7 +22636,7 @@
       <c r="AG91" s="38"/>
       <c r="AH91" s="64"/>
     </row>
-    <row r="92" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H92" s="37"/>
       <c r="K92" s="3"/>
       <c r="L92" s="3"/>
@@ -22642,7 +22650,7 @@
       <c r="AG92" s="38"/>
       <c r="AH92" s="64"/>
     </row>
-    <row r="93" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H93" s="37"/>
       <c r="K93" s="3"/>
       <c r="L93" s="3"/>
@@ -22656,7 +22664,7 @@
       <c r="AG93" s="38"/>
       <c r="AH93" s="64"/>
     </row>
-    <row r="94" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H94" s="37"/>
       <c r="K94" s="3"/>
       <c r="L94" s="3"/>
@@ -22670,7 +22678,7 @@
       <c r="AG94" s="38"/>
       <c r="AH94" s="64"/>
     </row>
-    <row r="95" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H95" s="37"/>
       <c r="K95" s="3"/>
       <c r="L95" s="3"/>
@@ -22684,7 +22692,7 @@
       <c r="AG95" s="38"/>
       <c r="AH95" s="64"/>
     </row>
-    <row r="96" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H96" s="37"/>
       <c r="K96" s="3"/>
       <c r="L96" s="3"/>
@@ -22698,7 +22706,7 @@
       <c r="AG96" s="38"/>
       <c r="AH96" s="64"/>
     </row>
-    <row r="97" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H97" s="37"/>
       <c r="K97" s="3"/>
       <c r="L97" s="3"/>
@@ -22712,7 +22720,7 @@
       <c r="AG97" s="38"/>
       <c r="AH97" s="64"/>
     </row>
-    <row r="98" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H98" s="37"/>
       <c r="K98" s="3"/>
       <c r="L98" s="3"/>
@@ -22726,7 +22734,7 @@
       <c r="AG98" s="38"/>
       <c r="AH98" s="64"/>
     </row>
-    <row r="99" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H99" s="37"/>
       <c r="K99" s="3"/>
       <c r="L99" s="3"/>
@@ -22741,7 +22749,7 @@
       <c r="AH99" s="64"/>
       <c r="BF99" s="68"/>
     </row>
-    <row r="100" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H100" s="37"/>
       <c r="K100" s="3"/>
       <c r="L100" s="3"/>
@@ -22756,7 +22764,7 @@
       <c r="AH100" s="64"/>
       <c r="BF100" s="68"/>
     </row>
-    <row r="101" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H101" s="37"/>
       <c r="K101" s="3"/>
       <c r="L101" s="3"/>
@@ -22771,7 +22779,7 @@
       <c r="AH101" s="64"/>
       <c r="BF101" s="68"/>
     </row>
-    <row r="102" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H102" s="37"/>
       <c r="K102" s="3"/>
       <c r="L102" s="3"/>
@@ -22786,7 +22794,7 @@
       <c r="AH102" s="64"/>
       <c r="BF102" s="68"/>
     </row>
-    <row r="103" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H103" s="37"/>
       <c r="K103" s="3"/>
       <c r="L103" s="3"/>
@@ -22801,7 +22809,7 @@
       <c r="AH103" s="64"/>
       <c r="BF103" s="68"/>
     </row>
-    <row r="104" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H104" s="37"/>
       <c r="K104" s="3"/>
       <c r="L104" s="3"/>
@@ -22816,7 +22824,7 @@
       <c r="AH104" s="64"/>
       <c r="BF104" s="68"/>
     </row>
-    <row r="105" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H105" s="37"/>
       <c r="K105" s="3"/>
       <c r="L105" s="3"/>
@@ -22831,7 +22839,7 @@
       <c r="AH105" s="64"/>
       <c r="BF105" s="68"/>
     </row>
-    <row r="106" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H106" s="37"/>
       <c r="K106" s="3"/>
       <c r="L106" s="3"/>
@@ -22846,7 +22854,7 @@
       <c r="AH106" s="64"/>
       <c r="BF106" s="68"/>
     </row>
-    <row r="107" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H107" s="37"/>
       <c r="K107" s="3"/>
       <c r="L107" s="3"/>
@@ -22861,7 +22869,7 @@
       <c r="AH107" s="64"/>
       <c r="BF107" s="68"/>
     </row>
-    <row r="108" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H108" s="37"/>
       <c r="K108" s="3"/>
       <c r="L108" s="3"/>
@@ -22876,7 +22884,7 @@
       <c r="AH108" s="64"/>
       <c r="BF108" s="68"/>
     </row>
-    <row r="109" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H109" s="37"/>
       <c r="K109" s="3"/>
       <c r="L109" s="3"/>
@@ -22891,7 +22899,7 @@
       <c r="AH109" s="64"/>
       <c r="BF109" s="68"/>
     </row>
-    <row r="110" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H110" s="37"/>
       <c r="K110" s="3"/>
       <c r="L110" s="3"/>
@@ -22906,7 +22914,7 @@
       <c r="AH110" s="64"/>
       <c r="BF110" s="68"/>
     </row>
-    <row r="111" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H111" s="37"/>
       <c r="K111" s="3"/>
       <c r="L111" s="3"/>
@@ -22921,7 +22929,7 @@
       <c r="AH111" s="64"/>
       <c r="BF111" s="68"/>
     </row>
-    <row r="112" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H112" s="37"/>
       <c r="K112" s="3"/>
       <c r="L112" s="3"/>
@@ -22936,7 +22944,7 @@
       <c r="AH112" s="64"/>
       <c r="BF112" s="68"/>
     </row>
-    <row r="113" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H113" s="37"/>
       <c r="K113" s="3"/>
       <c r="L113" s="3"/>
@@ -22951,7 +22959,7 @@
       <c r="AH113" s="64"/>
       <c r="BF113" s="68"/>
     </row>
-    <row r="114" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H114" s="37"/>
       <c r="K114" s="3"/>
       <c r="L114" s="3"/>
@@ -22966,7 +22974,7 @@
       <c r="AH114" s="64"/>
       <c r="BF114" s="68"/>
     </row>
-    <row r="115" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H115" s="37"/>
       <c r="K115" s="3"/>
       <c r="L115" s="3"/>
@@ -22981,7 +22989,7 @@
       <c r="AH115" s="64"/>
       <c r="BF115" s="68"/>
     </row>
-    <row r="116" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H116" s="37"/>
       <c r="K116" s="3"/>
       <c r="L116" s="3"/>
@@ -22992,7 +23000,7 @@
       <c r="AD116" s="6"/>
       <c r="AG116" s="38"/>
     </row>
-    <row r="117" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H117" s="37"/>
       <c r="K117" s="3"/>
       <c r="L117" s="3"/>
@@ -23003,7 +23011,7 @@
       <c r="AD117" s="72"/>
       <c r="AG117" s="38"/>
     </row>
-    <row r="118" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H118" s="37"/>
       <c r="K118" s="3"/>
       <c r="L118" s="3"/>
@@ -23018,7 +23026,7 @@
       <c r="AH118" s="64"/>
       <c r="BF118" s="68"/>
     </row>
-    <row r="119" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H119" s="37"/>
       <c r="K119" s="3"/>
       <c r="L119" s="3"/>
@@ -23033,7 +23041,7 @@
       <c r="AH119" s="64"/>
       <c r="BF119" s="68"/>
     </row>
-    <row r="120" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H120" s="37"/>
       <c r="K120" s="3"/>
       <c r="L120" s="3"/>
@@ -23048,7 +23056,7 @@
       <c r="AH120" s="64"/>
       <c r="BF120" s="68"/>
     </row>
-    <row r="121" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H121" s="37"/>
       <c r="K121" s="3"/>
       <c r="L121" s="3"/>
@@ -23060,7 +23068,7 @@
       <c r="AG121" s="38"/>
       <c r="BF121" s="68"/>
     </row>
-    <row r="122" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H122" s="37"/>
       <c r="K122" s="3"/>
       <c r="L122" s="3"/>
@@ -23075,7 +23083,7 @@
       <c r="AH122" s="64"/>
       <c r="BF122" s="68"/>
     </row>
-    <row r="123" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H123" s="37"/>
       <c r="K123" s="3"/>
       <c r="L123" s="3"/>
@@ -23090,7 +23098,7 @@
       <c r="AH123" s="64"/>
       <c r="BF123" s="68"/>
     </row>
-    <row r="124" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H124" s="37"/>
       <c r="K124" s="3"/>
       <c r="L124" s="3"/>
@@ -23105,7 +23113,7 @@
       <c r="AH124" s="64"/>
       <c r="BF124" s="68"/>
     </row>
-    <row r="125" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H125" s="37"/>
       <c r="K125" s="3"/>
       <c r="L125" s="3"/>
@@ -23117,7 +23125,7 @@
       <c r="AG125" s="38"/>
       <c r="BF125" s="68"/>
     </row>
-    <row r="126" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H126" s="37"/>
       <c r="K126" s="3"/>
       <c r="L126" s="3"/>
@@ -23129,7 +23137,7 @@
       <c r="AG126" s="38"/>
       <c r="BF126" s="68"/>
     </row>
-    <row r="127" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H127" s="37"/>
       <c r="K127" s="3"/>
       <c r="L127" s="3"/>
@@ -23141,7 +23149,7 @@
       <c r="AG127" s="38"/>
       <c r="BF127" s="68"/>
     </row>
-    <row r="128" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H128" s="37"/>
       <c r="K128" s="3"/>
       <c r="L128" s="3"/>
@@ -23159,7 +23167,7 @@
       <c r="BF128" s="68"/>
       <c r="BP128" s="10"/>
     </row>
-    <row r="129" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H129" s="37"/>
       <c r="K129" s="3"/>
       <c r="L129" s="3"/>
@@ -23176,7 +23184,7 @@
       <c r="BF129" s="68"/>
       <c r="BP129" s="10"/>
     </row>
-    <row r="130" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H130" s="37"/>
       <c r="K130" s="3"/>
       <c r="L130" s="3"/>
@@ -23193,7 +23201,7 @@
       <c r="BF130" s="68"/>
       <c r="BP130" s="10"/>
     </row>
-    <row r="131" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H131" s="37"/>
       <c r="K131" s="3"/>
       <c r="L131" s="3"/>
@@ -23210,7 +23218,7 @@
       <c r="BF131" s="68"/>
       <c r="BP131" s="10"/>
     </row>
-    <row r="132" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H132" s="37"/>
       <c r="K132" s="3"/>
       <c r="L132" s="3"/>
@@ -23227,7 +23235,7 @@
       <c r="BF132" s="68"/>
       <c r="BP132" s="10"/>
     </row>
-    <row r="133" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H133" s="37"/>
       <c r="K133" s="3"/>
       <c r="L133" s="3"/>
@@ -23244,7 +23252,7 @@
       <c r="BF133" s="68"/>
       <c r="BP133" s="10"/>
     </row>
-    <row r="134" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H134" s="37"/>
       <c r="K134" s="3"/>
       <c r="L134" s="3"/>
@@ -23261,7 +23269,7 @@
       <c r="BF134" s="68"/>
       <c r="BP134" s="10"/>
     </row>
-    <row r="135" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H135" s="37"/>
       <c r="K135" s="3"/>
       <c r="L135" s="3"/>
@@ -23277,7 +23285,7 @@
       <c r="AI135" s="38"/>
       <c r="BF135" s="68"/>
     </row>
-    <row r="136" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H136" s="37"/>
       <c r="K136" s="3"/>
       <c r="L136" s="3"/>
@@ -23293,7 +23301,7 @@
       <c r="AI136" s="38"/>
       <c r="BF136" s="68"/>
     </row>
-    <row r="137" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H137" s="37"/>
       <c r="K137" s="3"/>
       <c r="L137" s="3"/>
@@ -23309,7 +23317,7 @@
       <c r="AI137" s="38"/>
       <c r="BF137" s="68"/>
     </row>
-    <row r="138" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H138" s="37"/>
       <c r="K138" s="3"/>
       <c r="L138" s="3"/>
@@ -23325,7 +23333,7 @@
       <c r="AI138" s="38"/>
       <c r="BF138" s="68"/>
     </row>
-    <row r="139" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H139" s="37"/>
       <c r="K139" s="3"/>
       <c r="L139" s="3"/>
@@ -23341,7 +23349,7 @@
       <c r="AI139" s="38"/>
       <c r="BF139" s="68"/>
     </row>
-    <row r="140" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H140" s="37"/>
       <c r="K140" s="3"/>
       <c r="L140" s="3"/>
@@ -23357,7 +23365,7 @@
       <c r="AI140" s="38"/>
       <c r="BF140" s="68"/>
     </row>
-    <row r="141" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H141" s="37"/>
       <c r="K141" s="3"/>
       <c r="L141" s="3"/>
@@ -23373,7 +23381,7 @@
       <c r="AI141" s="38"/>
       <c r="BF141" s="68"/>
     </row>
-    <row r="142" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H142" s="37"/>
       <c r="K142" s="3"/>
       <c r="L142" s="3"/>
@@ -23389,7 +23397,7 @@
       <c r="AI142" s="38"/>
       <c r="BF142" s="68"/>
     </row>
-    <row r="143" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H143" s="37"/>
       <c r="K143" s="3"/>
       <c r="L143" s="3"/>
@@ -23405,7 +23413,7 @@
       <c r="AI143" s="38"/>
       <c r="BF143" s="68"/>
     </row>
-    <row r="144" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H144" s="37"/>
       <c r="K144" s="3"/>
       <c r="L144" s="3"/>
@@ -23421,7 +23429,7 @@
       <c r="AI144" s="38"/>
       <c r="BF144" s="68"/>
     </row>
-    <row r="145" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H145" s="37"/>
       <c r="K145" s="3"/>
       <c r="L145" s="3"/>
@@ -23437,7 +23445,7 @@
       <c r="AI145" s="38"/>
       <c r="BF145" s="68"/>
     </row>
-    <row r="146" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H146" s="37"/>
       <c r="K146" s="3"/>
       <c r="L146" s="3"/>
@@ -23453,7 +23461,7 @@
       <c r="AI146" s="38"/>
       <c r="BF146" s="68"/>
     </row>
-    <row r="147" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H147" s="37"/>
       <c r="K147" s="3"/>
       <c r="L147" s="3"/>
@@ -23469,7 +23477,7 @@
       <c r="AI147" s="38"/>
       <c r="BF147" s="68"/>
     </row>
-    <row r="148" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H148" s="37"/>
       <c r="K148" s="3"/>
       <c r="L148" s="3"/>
@@ -23485,7 +23493,7 @@
       <c r="AI148" s="38"/>
       <c r="BF148" s="68"/>
     </row>
-    <row r="149" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H149" s="37"/>
       <c r="K149" s="3"/>
       <c r="L149" s="3"/>
@@ -23501,7 +23509,7 @@
       <c r="AI149" s="38"/>
       <c r="BF149" s="68"/>
     </row>
-    <row r="150" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H150" s="37"/>
       <c r="K150" s="3"/>
       <c r="L150" s="3"/>
@@ -23517,7 +23525,7 @@
       <c r="AI150" s="38"/>
       <c r="BF150" s="68"/>
     </row>
-    <row r="151" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H151" s="37"/>
       <c r="K151" s="3"/>
       <c r="L151" s="3"/>
@@ -23533,7 +23541,7 @@
       <c r="AI151" s="38"/>
       <c r="BF151" s="68"/>
     </row>
-    <row r="152" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H152" s="37"/>
       <c r="K152" s="3"/>
       <c r="L152" s="3"/>
@@ -23549,7 +23557,7 @@
       <c r="AI152" s="38"/>
       <c r="BF152" s="68"/>
     </row>
-    <row r="153" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H153" s="37"/>
       <c r="K153" s="3"/>
       <c r="L153" s="3"/>
@@ -23565,7 +23573,7 @@
       <c r="AI153" s="38"/>
       <c r="BF153" s="68"/>
     </row>
-    <row r="154" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H154" s="37"/>
       <c r="K154" s="3"/>
       <c r="L154" s="3"/>
@@ -23581,7 +23589,7 @@
       <c r="AI154" s="38"/>
       <c r="BF154" s="68"/>
     </row>
-    <row r="155" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H155" s="37"/>
       <c r="K155" s="3"/>
       <c r="L155" s="3"/>
@@ -23597,7 +23605,7 @@
       <c r="AI155" s="38"/>
       <c r="BF155" s="68"/>
     </row>
-    <row r="156" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H156" s="37"/>
       <c r="K156" s="3"/>
       <c r="L156" s="3"/>
@@ -23613,7 +23621,7 @@
       <c r="AI156" s="38"/>
       <c r="BF156" s="68"/>
     </row>
-    <row r="157" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H157" s="37"/>
       <c r="K157" s="3"/>
       <c r="L157" s="3"/>
@@ -23629,7 +23637,7 @@
       <c r="AI157" s="38"/>
       <c r="BF157" s="68"/>
     </row>
-    <row r="158" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H158" s="37"/>
       <c r="K158" s="3"/>
       <c r="L158" s="3"/>
@@ -23645,7 +23653,7 @@
       <c r="AI158" s="38"/>
       <c r="BF158" s="68"/>
     </row>
-    <row r="159" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H159" s="37"/>
       <c r="K159" s="3"/>
       <c r="L159" s="3"/>
@@ -23661,7 +23669,7 @@
       <c r="AI159" s="38"/>
       <c r="BF159" s="68"/>
     </row>
-    <row r="160" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H160" s="37"/>
       <c r="K160" s="3"/>
       <c r="L160" s="3"/>
@@ -23677,7 +23685,7 @@
       <c r="AI160" s="38"/>
       <c r="BF160" s="68"/>
     </row>
-    <row r="161" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H161" s="37"/>
       <c r="K161" s="3"/>
       <c r="L161" s="3"/>
@@ -23693,7 +23701,7 @@
       <c r="AI161" s="38"/>
       <c r="BF161" s="68"/>
     </row>
-    <row r="162" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H162" s="37"/>
       <c r="K162" s="3"/>
       <c r="L162" s="3"/>
@@ -23709,7 +23717,7 @@
       <c r="AI162" s="38"/>
       <c r="BF162" s="68"/>
     </row>
-    <row r="163" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H163" s="37"/>
       <c r="K163" s="3"/>
       <c r="L163" s="3"/>
@@ -23725,7 +23733,7 @@
       <c r="AI163" s="38"/>
       <c r="BF163" s="68"/>
     </row>
-    <row r="164" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H164" s="37"/>
       <c r="K164" s="3"/>
       <c r="L164" s="3"/>
@@ -23740,7 +23748,7 @@
       <c r="AI164" s="38"/>
       <c r="BF164" s="68"/>
     </row>
-    <row r="165" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H165" s="37"/>
       <c r="K165" s="3"/>
       <c r="L165" s="3"/>
@@ -23755,7 +23763,7 @@
       <c r="AI165" s="38"/>
       <c r="BF165" s="68"/>
     </row>
-    <row r="166" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H166" s="37"/>
       <c r="K166" s="3"/>
       <c r="L166" s="3"/>
@@ -23771,7 +23779,7 @@
       <c r="AJ166" s="38"/>
       <c r="BF166" s="68"/>
     </row>
-    <row r="167" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H167" s="37"/>
       <c r="K167" s="3"/>
       <c r="L167" s="3"/>
@@ -23786,7 +23794,7 @@
       <c r="AI167" s="38"/>
       <c r="BF167" s="68"/>
     </row>
-    <row r="168" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H168" s="37"/>
       <c r="K168" s="3"/>
       <c r="L168" s="3"/>
@@ -23801,7 +23809,7 @@
       <c r="AI168" s="38"/>
       <c r="BF168" s="68"/>
     </row>
-    <row r="169" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H169" s="37"/>
       <c r="K169" s="3"/>
       <c r="L169" s="3"/>
@@ -23816,7 +23824,7 @@
       <c r="AI169" s="38"/>
       <c r="BF169" s="68"/>
     </row>
-    <row r="170" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H170" s="37"/>
       <c r="K170" s="3"/>
       <c r="L170" s="3"/>
@@ -23831,7 +23839,7 @@
       <c r="AI170" s="38"/>
       <c r="BF170" s="68"/>
     </row>
-    <row r="171" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H171" s="37"/>
       <c r="K171" s="3"/>
       <c r="L171" s="3"/>
@@ -23846,7 +23854,7 @@
       <c r="AI171" s="38"/>
       <c r="BF171" s="68"/>
     </row>
-    <row r="172" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H172" s="37"/>
       <c r="K172" s="3"/>
       <c r="L172" s="3"/>
@@ -23861,7 +23869,7 @@
       <c r="AI172" s="38"/>
       <c r="BF172" s="68"/>
     </row>
-    <row r="173" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H173" s="37"/>
       <c r="K173" s="3"/>
       <c r="L173" s="3"/>
@@ -23876,7 +23884,7 @@
       <c r="AI173" s="38"/>
       <c r="BF173" s="68"/>
     </row>
-    <row r="174" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H174" s="37"/>
       <c r="K174" s="3"/>
       <c r="L174" s="3"/>
@@ -23891,7 +23899,7 @@
       <c r="AI174" s="38"/>
       <c r="BF174" s="68"/>
     </row>
-    <row r="175" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H175" s="37"/>
       <c r="K175" s="3"/>
       <c r="L175" s="3"/>
@@ -23906,7 +23914,7 @@
       <c r="AI175" s="38"/>
       <c r="BF175" s="68"/>
     </row>
-    <row r="176" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H176" s="37"/>
       <c r="K176" s="3"/>
       <c r="L176" s="3"/>
@@ -23921,7 +23929,7 @@
       <c r="AI176" s="38"/>
       <c r="BF176" s="68"/>
     </row>
-    <row r="177" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H177" s="37"/>
       <c r="K177" s="3"/>
       <c r="L177" s="3"/>
@@ -23936,7 +23944,7 @@
       <c r="AI177" s="38"/>
       <c r="BF177" s="68"/>
     </row>
-    <row r="178" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H178" s="37"/>
       <c r="K178" s="3"/>
       <c r="L178" s="3"/>
@@ -23951,7 +23959,7 @@
       <c r="AI178" s="38"/>
       <c r="BF178" s="68"/>
     </row>
-    <row r="179" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H179" s="37"/>
       <c r="K179" s="3"/>
       <c r="L179" s="3"/>
@@ -23966,7 +23974,7 @@
       <c r="AI179" s="38"/>
       <c r="BF179" s="68"/>
     </row>
-    <row r="180" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H180" s="37"/>
       <c r="K180" s="3"/>
       <c r="L180" s="3"/>
@@ -23981,7 +23989,7 @@
       <c r="AI180" s="38"/>
       <c r="BF180" s="68"/>
     </row>
-    <row r="181" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H181" s="37"/>
       <c r="K181" s="3"/>
       <c r="L181" s="3"/>
@@ -23996,7 +24004,7 @@
       <c r="AI181" s="38"/>
       <c r="BF181" s="68"/>
     </row>
-    <row r="182" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H182" s="37"/>
       <c r="K182" s="3"/>
       <c r="L182" s="3"/>
@@ -24011,7 +24019,7 @@
       <c r="AI182" s="38"/>
       <c r="BF182" s="68"/>
     </row>
-    <row r="183" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H183" s="37"/>
       <c r="K183" s="3"/>
       <c r="L183" s="3"/>
@@ -24026,7 +24034,7 @@
       <c r="AI183" s="38"/>
       <c r="BF183" s="68"/>
     </row>
-    <row r="184" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H184" s="37"/>
       <c r="K184" s="3"/>
       <c r="L184" s="3"/>
@@ -24041,7 +24049,7 @@
       <c r="AI184" s="38"/>
       <c r="BF184" s="68"/>
     </row>
-    <row r="185" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H185" s="37"/>
       <c r="K185" s="3"/>
       <c r="L185" s="3"/>
@@ -24056,7 +24064,7 @@
       <c r="AI185" s="38"/>
       <c r="BF185" s="68"/>
     </row>
-    <row r="186" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H186" s="37"/>
       <c r="K186" s="3"/>
       <c r="L186" s="3"/>
@@ -24071,7 +24079,7 @@
       <c r="AI186" s="38"/>
       <c r="BF186" s="68"/>
     </row>
-    <row r="187" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H187" s="37"/>
       <c r="K187" s="3"/>
       <c r="L187" s="3"/>
@@ -24086,7 +24094,7 @@
       <c r="AI187" s="38"/>
       <c r="BF187" s="68"/>
     </row>
-    <row r="188" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H188" s="37"/>
       <c r="K188" s="3"/>
       <c r="L188" s="3"/>
@@ -24101,7 +24109,7 @@
       <c r="AI188" s="38"/>
       <c r="BF188" s="68"/>
     </row>
-    <row r="189" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H189" s="37"/>
       <c r="K189" s="3"/>
       <c r="L189" s="3"/>
@@ -24116,7 +24124,7 @@
       <c r="AI189" s="38"/>
       <c r="BF189" s="68"/>
     </row>
-    <row r="190" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H190" s="37"/>
       <c r="K190" s="3"/>
       <c r="L190" s="3"/>
@@ -24128,7 +24136,7 @@
       <c r="AG190" s="38"/>
       <c r="AH190" s="64"/>
     </row>
-    <row r="191" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H191" s="37"/>
       <c r="K191" s="3"/>
       <c r="L191" s="3"/>
@@ -24141,7 +24149,7 @@
       <c r="AG191" s="38"/>
       <c r="AH191" s="64"/>
     </row>
-    <row r="192" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H192" s="37"/>
       <c r="K192" s="3"/>
       <c r="L192" s="3"/>
@@ -24155,7 +24163,7 @@
       <c r="AH192" s="64"/>
       <c r="BF192" s="68"/>
     </row>
-    <row r="193" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H193" s="37"/>
       <c r="K193" s="3"/>
       <c r="L193" s="3"/>

</xml_diff>

<commit_message>
Reporte de liquidacion asistencia en proceso. Falta filtro proveedor y ajustar formato de pdf generado.
</commit_message>
<xml_diff>
--- a/Carga_Real_corto.xlsx
+++ b/Carga_Real_corto.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ON" sheetId="1" state="visible" r:id="rId3"/>
@@ -696,6 +696,7 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -717,6 +718,7 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -724,28 +726,33 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <strike val="true"/>
@@ -753,23 +760,27 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FFC9211E"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1496,6 +1507,7 @@
     <dxf>
       <font>
         <name val="Calibri"/>
+        <charset val="1"/>
         <family val="2"/>
         <b val="1"/>
         <i val="0"/>
@@ -1511,6 +1523,7 @@
     <dxf>
       <font>
         <name val="Calibri"/>
+        <charset val="1"/>
         <family val="2"/>
         <b val="1"/>
         <i val="0"/>
@@ -2123,7 +2136,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="2" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="37" t="s">
         <v>106</v>
       </c>
@@ -2135,7 +2148,7 @@
       </c>
       <c r="D2" s="39"/>
       <c r="E2" s="39" t="n">
-        <v>45612</v>
+        <v>45673</v>
       </c>
       <c r="F2" s="39" t="n">
         <v>45612</v>
@@ -2377,7 +2390,7 @@
       <c r="CU2" s="39"/>
       <c r="CV2" s="38"/>
     </row>
-    <row r="3" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
         <v>106</v>
       </c>
@@ -2389,7 +2402,7 @@
       </c>
       <c r="D3" s="39"/>
       <c r="E3" s="39" t="n">
-        <v>45612</v>
+        <v>45673</v>
       </c>
       <c r="F3" s="39" t="n">
         <v>45612</v>
@@ -2571,7 +2584,7 @@
       <c r="CU3" s="39"/>
       <c r="CV3" s="38"/>
     </row>
-    <row r="4" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="37" t="s">
         <v>106</v>
       </c>
@@ -2583,7 +2596,7 @@
       </c>
       <c r="D4" s="39"/>
       <c r="E4" s="39" t="n">
-        <v>45612</v>
+        <v>45673</v>
       </c>
       <c r="F4" s="39" t="n">
         <v>45612</v>
@@ -2807,7 +2820,7 @@
       <c r="CU4" s="39"/>
       <c r="CV4" s="38"/>
     </row>
-    <row r="5" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="37"/>
       <c r="B5" s="38"/>
       <c r="C5" s="38"/>
@@ -2909,7 +2922,7 @@
       <c r="CU5" s="39"/>
       <c r="CV5" s="38"/>
     </row>
-    <row r="6" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="37"/>
       <c r="B6" s="38"/>
       <c r="C6" s="38"/>
@@ -3011,7 +3024,7 @@
       <c r="CU6" s="39"/>
       <c r="CV6" s="38"/>
     </row>
-    <row r="7" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="37"/>
       <c r="B7" s="38"/>
       <c r="C7" s="38"/>
@@ -3113,7 +3126,7 @@
       <c r="CU7" s="39"/>
       <c r="CV7" s="38"/>
     </row>
-    <row r="8" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="37"/>
       <c r="B8" s="38"/>
       <c r="C8" s="38"/>
@@ -3215,7 +3228,7 @@
       <c r="CU8" s="39"/>
       <c r="CV8" s="38"/>
     </row>
-    <row r="9" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="37"/>
       <c r="B9" s="38"/>
       <c r="C9" s="38"/>
@@ -3317,7 +3330,7 @@
       <c r="CU9" s="39"/>
       <c r="CV9" s="38"/>
     </row>
-    <row r="10" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="37"/>
       <c r="B10" s="38"/>
       <c r="C10" s="38"/>
@@ -3419,7 +3432,7 @@
       <c r="CU10" s="39"/>
       <c r="CV10" s="38"/>
     </row>
-    <row r="11" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="37"/>
       <c r="B11" s="38"/>
       <c r="C11" s="38"/>
@@ -3521,7 +3534,7 @@
       <c r="CU11" s="39"/>
       <c r="CV11" s="38"/>
     </row>
-    <row r="12" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="37"/>
       <c r="B12" s="38"/>
       <c r="C12" s="38"/>
@@ -3623,7 +3636,7 @@
       <c r="CU12" s="39"/>
       <c r="CV12" s="38"/>
     </row>
-    <row r="13" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="37"/>
       <c r="B13" s="38"/>
       <c r="C13" s="38"/>
@@ -3725,7 +3738,7 @@
       <c r="CU13" s="39"/>
       <c r="CV13" s="38"/>
     </row>
-    <row r="14" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="37"/>
       <c r="B14" s="38"/>
       <c r="C14" s="38"/>
@@ -3827,7 +3840,7 @@
       <c r="CU14" s="39"/>
       <c r="CV14" s="38"/>
     </row>
-    <row r="15" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="37"/>
       <c r="B15" s="38"/>
       <c r="C15" s="38"/>
@@ -3929,7 +3942,7 @@
       <c r="CU15" s="39"/>
       <c r="CV15" s="38"/>
     </row>
-    <row r="16" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="37"/>
       <c r="B16" s="38"/>
       <c r="C16" s="38"/>
@@ -4031,7 +4044,7 @@
       <c r="CU16" s="39"/>
       <c r="CV16" s="38"/>
     </row>
-    <row r="17" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="37"/>
       <c r="B17" s="38"/>
       <c r="C17" s="38"/>
@@ -4133,7 +4146,7 @@
       <c r="CU17" s="39"/>
       <c r="CV17" s="38"/>
     </row>
-    <row r="18" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="37"/>
       <c r="B18" s="38"/>
       <c r="C18" s="38"/>
@@ -4235,7 +4248,7 @@
       <c r="CU18" s="39"/>
       <c r="CV18" s="38"/>
     </row>
-    <row r="19" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="37"/>
       <c r="B19" s="38"/>
       <c r="C19" s="38"/>
@@ -4337,7 +4350,7 @@
       <c r="CU19" s="39"/>
       <c r="CV19" s="38"/>
     </row>
-    <row r="20" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="37"/>
       <c r="B20" s="38"/>
       <c r="C20" s="38"/>
@@ -4439,7 +4452,7 @@
       <c r="CU20" s="39"/>
       <c r="CV20" s="38"/>
     </row>
-    <row r="21" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="37"/>
       <c r="B21" s="38"/>
       <c r="C21" s="38"/>
@@ -4541,7 +4554,7 @@
       <c r="CU21" s="39"/>
       <c r="CV21" s="38"/>
     </row>
-    <row r="22" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="37"/>
       <c r="B22" s="38"/>
       <c r="C22" s="38"/>
@@ -4643,7 +4656,7 @@
       <c r="CU22" s="39"/>
       <c r="CV22" s="38"/>
     </row>
-    <row r="23" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="37"/>
       <c r="B23" s="38"/>
       <c r="C23" s="38"/>
@@ -4745,7 +4758,7 @@
       <c r="CU23" s="39"/>
       <c r="CV23" s="38"/>
     </row>
-    <row r="24" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="37"/>
       <c r="B24" s="38"/>
       <c r="C24" s="38"/>
@@ -4847,7 +4860,7 @@
       <c r="CU24" s="39"/>
       <c r="CV24" s="38"/>
     </row>
-    <row r="25" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="37"/>
       <c r="B25" s="38"/>
       <c r="C25" s="38"/>
@@ -4949,7 +4962,7 @@
       <c r="CU25" s="39"/>
       <c r="CV25" s="38"/>
     </row>
-    <row r="26" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="37"/>
       <c r="B26" s="38"/>
       <c r="C26" s="38"/>
@@ -5051,7 +5064,7 @@
       <c r="CU26" s="39"/>
       <c r="CV26" s="38"/>
     </row>
-    <row r="27" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="37"/>
       <c r="B27" s="38"/>
       <c r="C27" s="38"/>
@@ -5153,7 +5166,7 @@
       <c r="CU27" s="39"/>
       <c r="CV27" s="38"/>
     </row>
-    <row r="28" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="37"/>
       <c r="B28" s="38"/>
       <c r="C28" s="38"/>
@@ -5255,7 +5268,7 @@
       <c r="CU28" s="39"/>
       <c r="CV28" s="38"/>
     </row>
-    <row r="29" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="37"/>
       <c r="B29" s="38"/>
       <c r="C29" s="38"/>
@@ -5357,7 +5370,7 @@
       <c r="CU29" s="39"/>
       <c r="CV29" s="38"/>
     </row>
-    <row r="30" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="37"/>
       <c r="B30" s="38"/>
       <c r="C30" s="38"/>
@@ -5459,7 +5472,7 @@
       <c r="CU30" s="39"/>
       <c r="CV30" s="38"/>
     </row>
-    <row r="31" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="37"/>
       <c r="B31" s="38"/>
       <c r="C31" s="38"/>
@@ -5561,7 +5574,7 @@
       <c r="CU31" s="39"/>
       <c r="CV31" s="38"/>
     </row>
-    <row r="32" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="37"/>
       <c r="B32" s="38"/>
       <c r="C32" s="38"/>
@@ -5662,7 +5675,7 @@
       <c r="CU32" s="39"/>
       <c r="CV32" s="38"/>
     </row>
-    <row r="33" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="37"/>
       <c r="B33" s="38"/>
       <c r="C33" s="38"/>
@@ -5763,7 +5776,7 @@
       <c r="CU33" s="39"/>
       <c r="CV33" s="38"/>
     </row>
-    <row r="34" s="59" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" s="59" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="50"/>
       <c r="B34" s="51"/>
       <c r="C34" s="51"/>
@@ -5864,7 +5877,7 @@
       <c r="CU34" s="52"/>
       <c r="CV34" s="51"/>
     </row>
-    <row r="35" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="37"/>
       <c r="B35" s="38"/>
       <c r="C35" s="38"/>
@@ -5965,7 +5978,7 @@
       <c r="CU35" s="39"/>
       <c r="CV35" s="38"/>
     </row>
-    <row r="36" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="37"/>
       <c r="B36" s="38"/>
       <c r="C36" s="38"/>
@@ -6072,7 +6085,7 @@
       <c r="DA36" s="39"/>
       <c r="DB36" s="38"/>
     </row>
-    <row r="37" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="37"/>
       <c r="B37" s="38"/>
       <c r="C37" s="38"/>
@@ -6179,7 +6192,7 @@
       <c r="DA37" s="39"/>
       <c r="DB37" s="38"/>
     </row>
-    <row r="38" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="37"/>
       <c r="B38" s="38"/>
       <c r="C38" s="38"/>
@@ -6286,7 +6299,7 @@
       <c r="DA38" s="39"/>
       <c r="DB38" s="38"/>
     </row>
-    <row r="39" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="37"/>
       <c r="B39" s="38"/>
       <c r="C39" s="38"/>
@@ -6393,7 +6406,7 @@
       <c r="DA39" s="39"/>
       <c r="DB39" s="38"/>
     </row>
-    <row r="40" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="37"/>
       <c r="B40" s="38"/>
       <c r="C40" s="38"/>
@@ -6500,7 +6513,7 @@
       <c r="DA40" s="39"/>
       <c r="DB40" s="38"/>
     </row>
-    <row r="41" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="37"/>
       <c r="B41" s="38"/>
       <c r="C41" s="38"/>
@@ -6607,7 +6620,7 @@
       <c r="DA41" s="39"/>
       <c r="DB41" s="38"/>
     </row>
-    <row r="42" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="37"/>
       <c r="B42" s="38"/>
       <c r="C42" s="38"/>
@@ -6709,7 +6722,7 @@
       <c r="CU42" s="39"/>
       <c r="CV42" s="38"/>
     </row>
-    <row r="43" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="37"/>
       <c r="B43" s="38"/>
       <c r="C43" s="38"/>
@@ -6811,7 +6824,7 @@
       <c r="CU43" s="39"/>
       <c r="CV43" s="38"/>
     </row>
-    <row r="44" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="37"/>
       <c r="B44" s="38"/>
       <c r="C44" s="38"/>
@@ -6913,7 +6926,7 @@
       <c r="CU44" s="39"/>
       <c r="CV44" s="38"/>
     </row>
-    <row r="45" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="37"/>
       <c r="B45" s="38"/>
       <c r="C45" s="38"/>
@@ -7015,7 +7028,7 @@
       <c r="CU45" s="39"/>
       <c r="CV45" s="38"/>
     </row>
-    <row r="46" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="37"/>
       <c r="B46" s="38"/>
       <c r="C46" s="38"/>
@@ -7117,7 +7130,7 @@
       <c r="CU46" s="39"/>
       <c r="CV46" s="38"/>
     </row>
-    <row r="47" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="37"/>
       <c r="B47" s="38"/>
       <c r="C47" s="38"/>
@@ -7219,7 +7232,7 @@
       <c r="CU47" s="39"/>
       <c r="CV47" s="38"/>
     </row>
-    <row r="48" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="37"/>
       <c r="B48" s="38"/>
       <c r="C48" s="38"/>
@@ -7321,7 +7334,7 @@
       <c r="CU48" s="39"/>
       <c r="CV48" s="38"/>
     </row>
-    <row r="49" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="37"/>
       <c r="B49" s="38"/>
       <c r="C49" s="38"/>
@@ -7423,7 +7436,7 @@
       <c r="CU49" s="39"/>
       <c r="CV49" s="38"/>
     </row>
-    <row r="50" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="37"/>
       <c r="B50" s="38"/>
       <c r="C50" s="38"/>
@@ -7525,7 +7538,7 @@
       <c r="CU50" s="39"/>
       <c r="CV50" s="38"/>
     </row>
-    <row r="51" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="37"/>
       <c r="B51" s="38"/>
       <c r="C51" s="38"/>
@@ -7627,7 +7640,7 @@
       <c r="CU51" s="39"/>
       <c r="CV51" s="38"/>
     </row>
-    <row r="52" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" s="44" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="37"/>
       <c r="B52" s="38"/>
       <c r="C52" s="38"/>
@@ -7729,7 +7742,7 @@
       <c r="CU52" s="39"/>
       <c r="CV52" s="38"/>
     </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="37"/>
       <c r="B53" s="62"/>
       <c r="C53" s="62"/>
@@ -7825,7 +7838,7 @@
       <c r="CU53" s="63"/>
       <c r="CV53" s="62"/>
     </row>
-    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="37"/>
       <c r="B54" s="62"/>
       <c r="C54" s="62"/>
@@ -7921,7 +7934,7 @@
       <c r="CU54" s="63"/>
       <c r="CV54" s="62"/>
     </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="37"/>
       <c r="B55" s="62"/>
       <c r="C55" s="62"/>
@@ -8017,7 +8030,7 @@
       <c r="CU55" s="63"/>
       <c r="CV55" s="62"/>
     </row>
-    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="37"/>
       <c r="B56" s="62"/>
       <c r="C56" s="62"/>
@@ -8113,7 +8126,7 @@
       <c r="CU56" s="63"/>
       <c r="CV56" s="62"/>
     </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="37"/>
       <c r="B57" s="62"/>
       <c r="C57" s="62"/>
@@ -8209,7 +8222,7 @@
       <c r="CU57" s="63"/>
       <c r="CV57" s="62"/>
     </row>
-    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="62"/>
       <c r="C58" s="62"/>
       <c r="D58" s="63"/>
@@ -8304,7 +8317,7 @@
       <c r="CU58" s="63"/>
       <c r="CV58" s="62"/>
     </row>
-    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="62"/>
       <c r="C59" s="62"/>
       <c r="D59" s="63"/>
@@ -8399,7 +8412,7 @@
       <c r="CU59" s="63"/>
       <c r="CV59" s="62"/>
     </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="62"/>
       <c r="C60" s="62"/>
       <c r="D60" s="63"/>
@@ -8494,7 +8507,7 @@
       <c r="CU60" s="63"/>
       <c r="CV60" s="62"/>
     </row>
-    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="62"/>
       <c r="C61" s="62"/>
       <c r="D61" s="63"/>
@@ -8589,7 +8602,7 @@
       <c r="CU61" s="63"/>
       <c r="CV61" s="62"/>
     </row>
-    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="62"/>
       <c r="C62" s="38"/>
       <c r="D62" s="63"/>
@@ -8684,7 +8697,7 @@
       <c r="CU62" s="63"/>
       <c r="CV62" s="62"/>
     </row>
-    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="62"/>
       <c r="C63" s="38"/>
       <c r="D63" s="63"/>
@@ -8779,7 +8792,7 @@
       <c r="CU63" s="63"/>
       <c r="CV63" s="62"/>
     </row>
-    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="62"/>
       <c r="C64" s="38"/>
       <c r="D64" s="63"/>
@@ -8874,7 +8887,7 @@
       <c r="CU64" s="63"/>
       <c r="CV64" s="62"/>
     </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="62"/>
       <c r="C65" s="38"/>
       <c r="D65" s="63"/>
@@ -8972,7 +8985,7 @@
       <c r="CU65" s="63"/>
       <c r="CV65" s="62"/>
     </row>
-    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="62"/>
       <c r="C66" s="38"/>
       <c r="D66" s="62"/>
@@ -9069,7 +9082,7 @@
       <c r="CU66" s="63"/>
       <c r="CV66" s="62"/>
     </row>
-    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C67" s="38"/>
       <c r="E67" s="39"/>
       <c r="F67" s="39"/>
@@ -9102,7 +9115,7 @@
       <c r="CQ67" s="41"/>
       <c r="CR67" s="41"/>
     </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C68" s="38"/>
       <c r="E68" s="39"/>
       <c r="F68" s="39"/>
@@ -9133,7 +9146,7 @@
       <c r="CC68" s="39"/>
       <c r="CD68" s="42"/>
     </row>
-    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C69" s="38"/>
       <c r="E69" s="39"/>
       <c r="F69" s="39"/>
@@ -9164,7 +9177,7 @@
       <c r="CC69" s="39"/>
       <c r="CD69" s="42"/>
     </row>
-    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E70" s="39"/>
       <c r="F70" s="39"/>
       <c r="I70" s="38"/>
@@ -9193,7 +9206,7 @@
       <c r="CC70" s="39"/>
       <c r="CD70" s="42"/>
     </row>
-    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E71" s="39"/>
       <c r="F71" s="39"/>
       <c r="I71" s="38"/>
@@ -9224,7 +9237,7 @@
       <c r="CC71" s="39"/>
       <c r="CD71" s="42"/>
     </row>
-    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E72" s="39"/>
       <c r="F72" s="39"/>
       <c r="I72" s="38"/>
@@ -9253,7 +9266,7 @@
       <c r="CC72" s="39"/>
       <c r="CD72" s="42"/>
     </row>
-    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C73" s="38"/>
       <c r="E73" s="39"/>
       <c r="F73" s="39"/>
@@ -9285,7 +9298,7 @@
       <c r="CC73" s="39"/>
       <c r="CD73" s="42"/>
     </row>
-    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C74" s="38"/>
       <c r="E74" s="39"/>
       <c r="F74" s="39"/>
@@ -9317,7 +9330,7 @@
       <c r="CC74" s="39"/>
       <c r="CD74" s="42"/>
     </row>
-    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C75" s="38"/>
       <c r="E75" s="39"/>
       <c r="F75" s="39"/>
@@ -9349,7 +9362,7 @@
       <c r="CC75" s="39"/>
       <c r="CD75" s="42"/>
     </row>
-    <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C76" s="38"/>
       <c r="E76" s="39"/>
       <c r="F76" s="39"/>
@@ -9381,7 +9394,7 @@
       <c r="CC76" s="39"/>
       <c r="CD76" s="42"/>
     </row>
-    <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E77" s="39"/>
       <c r="F77" s="39"/>
       <c r="I77" s="38"/>
@@ -9412,7 +9425,7 @@
       <c r="CC77" s="39"/>
       <c r="CD77" s="42"/>
     </row>
-    <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E78" s="39"/>
       <c r="F78" s="39"/>
       <c r="I78" s="38"/>
@@ -9441,7 +9454,7 @@
       <c r="CC78" s="39"/>
       <c r="CD78" s="42"/>
     </row>
-    <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E79" s="39"/>
       <c r="F79" s="39"/>
       <c r="I79" s="38"/>
@@ -9470,7 +9483,7 @@
       <c r="CC79" s="39"/>
       <c r="CD79" s="42"/>
     </row>
-    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E80" s="39"/>
       <c r="F80" s="39"/>
       <c r="I80" s="38"/>
@@ -9499,7 +9512,7 @@
       <c r="CC80" s="39"/>
       <c r="CD80" s="42"/>
     </row>
-    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E81" s="39"/>
       <c r="F81" s="39"/>
       <c r="H81" s="72"/>
@@ -9527,7 +9540,7 @@
       <c r="CC81" s="39"/>
       <c r="CD81" s="42"/>
     </row>
-    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E82" s="39"/>
       <c r="F82" s="39"/>
       <c r="H82" s="72"/>
@@ -9555,7 +9568,7 @@
       <c r="CC82" s="39"/>
       <c r="CD82" s="42"/>
     </row>
-    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E83" s="39"/>
       <c r="F83" s="39"/>
       <c r="H83" s="72"/>
@@ -9583,7 +9596,7 @@
       <c r="CC83" s="39"/>
       <c r="CD83" s="42"/>
     </row>
-    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E84" s="39"/>
       <c r="F84" s="39"/>
       <c r="H84" s="72"/>
@@ -9611,7 +9624,7 @@
       <c r="CC84" s="39"/>
       <c r="CD84" s="42"/>
     </row>
-    <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E85" s="39"/>
       <c r="F85" s="39"/>
       <c r="H85" s="72"/>
@@ -9639,7 +9652,7 @@
       <c r="CC85" s="39"/>
       <c r="CD85" s="42"/>
     </row>
-    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E86" s="39"/>
       <c r="F86" s="39"/>
       <c r="H86" s="72"/>
@@ -9667,7 +9680,7 @@
       <c r="CC86" s="39"/>
       <c r="CD86" s="42"/>
     </row>
-    <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E87" s="39"/>
       <c r="F87" s="39"/>
       <c r="H87" s="72"/>
@@ -9695,7 +9708,7 @@
       <c r="CC87" s="39"/>
       <c r="CD87" s="42"/>
     </row>
-    <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E88" s="39"/>
       <c r="F88" s="39"/>
       <c r="H88" s="72"/>
@@ -9723,7 +9736,7 @@
       <c r="CC88" s="39"/>
       <c r="CD88" s="42"/>
     </row>
-    <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E89" s="39"/>
       <c r="F89" s="39"/>
       <c r="H89" s="72"/>
@@ -9750,7 +9763,7 @@
       <c r="CC89" s="39"/>
       <c r="CD89" s="42"/>
     </row>
-    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E90" s="39"/>
       <c r="F90" s="39"/>
       <c r="H90" s="72"/>
@@ -9777,7 +9790,7 @@
       <c r="CC90" s="39"/>
       <c r="CD90" s="42"/>
     </row>
-    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E91" s="39"/>
       <c r="F91" s="39"/>
       <c r="H91" s="72"/>
@@ -9804,7 +9817,7 @@
       <c r="CC91" s="39"/>
       <c r="CD91" s="42"/>
     </row>
-    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E92" s="39"/>
       <c r="F92" s="39"/>
       <c r="H92" s="72"/>
@@ -9831,7 +9844,7 @@
       <c r="CC92" s="39"/>
       <c r="CD92" s="42"/>
     </row>
-    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E93" s="39"/>
       <c r="F93" s="39"/>
       <c r="H93" s="72"/>
@@ -9857,7 +9870,7 @@
       <c r="CC93" s="39"/>
       <c r="CD93" s="42"/>
     </row>
-    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E94" s="39"/>
       <c r="F94" s="39"/>
       <c r="H94" s="72"/>
@@ -9883,7 +9896,7 @@
       <c r="CC94" s="39"/>
       <c r="CD94" s="42"/>
     </row>
-    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E95" s="39"/>
       <c r="F95" s="39"/>
       <c r="H95" s="72"/>
@@ -9909,7 +9922,7 @@
       <c r="CC95" s="39"/>
       <c r="CD95" s="42"/>
     </row>
-    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E96" s="39"/>
       <c r="F96" s="39"/>
       <c r="I96" s="38"/>
@@ -9932,7 +9945,7 @@
       <c r="CC96" s="39"/>
       <c r="CD96" s="42"/>
     </row>
-    <row r="97" s="87" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" s="87" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="74"/>
       <c r="B97" s="74"/>
       <c r="C97" s="74"/>
@@ -10034,7 +10047,7 @@
       <c r="CU97" s="86"/>
       <c r="CV97" s="74"/>
     </row>
-    <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E98" s="39"/>
       <c r="F98" s="39"/>
       <c r="I98" s="38"/>
@@ -10056,7 +10069,7 @@
       <c r="CC98" s="39"/>
       <c r="CD98" s="42"/>
     </row>
-    <row r="99" s="87" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" s="87" customFormat="true" ht="11.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="74"/>
       <c r="B99" s="74"/>
       <c r="C99" s="74"/>
@@ -18356,8 +18369,8 @@
       <c r="C2" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E2" s="61" t="n">
-        <v>45612</v>
+      <c r="E2" s="39" t="n">
+        <v>45673</v>
       </c>
       <c r="F2" s="61" t="n">
         <v>45612</v>
@@ -18483,8 +18496,8 @@
       <c r="C3" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E3" s="61" t="n">
-        <v>45612</v>
+      <c r="E3" s="39" t="n">
+        <v>45673</v>
       </c>
       <c r="F3" s="61" t="n">
         <v>45612</v>

</xml_diff>

<commit_message>
Procesamiento de Dataframe hoteles para dejarlo en formato excel inicial.
</commit_message>
<xml_diff>
--- a/Carga_Real_corto.xlsx
+++ b/Carga_Real_corto.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="216">
   <si>
     <t xml:space="preserve">Activo</t>
   </si>
@@ -218,7 +218,7 @@
     <t xml:space="preserve">Nombre Hotel 3</t>
   </si>
   <si>
-    <t xml:space="preserve">City_in_1</t>
+    <t xml:space="preserve">s</t>
   </si>
   <si>
     <t xml:space="preserve">Place_in_1</t>
@@ -578,6 +578,9 @@
     <t xml:space="preserve">Nacionalidad </t>
   </si>
   <si>
+    <t xml:space="preserve">City_in_1</t>
+  </si>
+  <si>
     <t xml:space="preserve">SI</t>
   </si>
   <si>
@@ -597,6 +600,9 @@
   </si>
   <si>
     <t xml:space="preserve">CHARTER WPU SCL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:30 12:15</t>
   </si>
   <si>
     <t xml:space="preserve">LA8097 SCL GRU</t>
@@ -630,9 +636,6 @@
   </si>
   <si>
     <t xml:space="preserve">HK30 WPU PUQ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:30 12:15</t>
   </si>
   <si>
     <t xml:space="preserve">LA94 PUQ SCL</t>
@@ -690,7 +693,7 @@
     <numFmt numFmtId="175" formatCode="@"/>
     <numFmt numFmtId="176" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -765,6 +768,14 @@
     <font>
       <sz val="8"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -889,7 +900,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="151">
+  <cellXfs count="152">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1382,6 +1393,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1398,15 +1413,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1422,27 +1437,27 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="176" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -18233,7 +18248,7 @@
         <v>63</v>
       </c>
       <c r="BA1" s="31" t="s">
-        <v>64</v>
+        <v>184</v>
       </c>
       <c r="BB1" s="31" t="s">
         <v>65</v>
@@ -18382,28 +18397,28 @@
         <v>110</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K2" s="93" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="M2" s="37" t="s">
         <v>114</v>
       </c>
       <c r="N2" s="44" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="O2" s="44" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="P2" s="93" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="Q2" s="61" t="n">
         <v>26176</v>
@@ -18421,21 +18436,26 @@
         <v>120</v>
       </c>
       <c r="V2" s="44" t="s">
-        <v>190</v>
-      </c>
-      <c r="W2" s="5"/>
+        <v>191</v>
+      </c>
+      <c r="W2" s="9" t="n">
+        <v>45614</v>
+      </c>
+      <c r="X2" s="123" t="s">
+        <v>192</v>
+      </c>
       <c r="Z2" s="9"/>
-      <c r="AA2" s="123"/>
-      <c r="AB2" s="124" t="s">
-        <v>191</v>
+      <c r="AA2" s="124"/>
+      <c r="AB2" s="125" t="s">
+        <v>193</v>
       </c>
       <c r="AC2" s="9" t="n">
         <v>45613</v>
       </c>
-      <c r="AD2" s="125" t="n">
+      <c r="AD2" s="126" t="n">
         <v>0.878472222222222</v>
       </c>
-      <c r="AE2" s="123"/>
+      <c r="AE2" s="124"/>
       <c r="AF2" s="64"/>
       <c r="AH2" s="64"/>
       <c r="AK2" s="92" t="n">
@@ -18447,7 +18467,7 @@
       <c r="AR2" s="5"/>
       <c r="AS2" s="5"/>
       <c r="AV2" s="10" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="AW2" s="5" t="n">
         <v>45612</v>
@@ -18459,7 +18479,7 @@
         <v>177</v>
       </c>
       <c r="AZ2" s="10" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="BA2" s="62"/>
       <c r="BB2" s="62"/>
@@ -18471,13 +18491,13 @@
       <c r="BH2" s="62"/>
       <c r="BI2" s="62"/>
       <c r="BJ2" s="62"/>
-      <c r="BL2" s="126"/>
+      <c r="BL2" s="127"/>
       <c r="BM2" s="62"/>
       <c r="BN2" s="63"/>
       <c r="BO2" s="62"/>
       <c r="BP2" s="62"/>
       <c r="BQ2" s="63"/>
-      <c r="BR2" s="126"/>
+      <c r="BR2" s="127"/>
       <c r="BS2" s="63"/>
       <c r="BT2" s="63"/>
       <c r="BU2" s="63"/>
@@ -18509,91 +18529,91 @@
         <v>110</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K3" s="93" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="M3" s="37" t="s">
         <v>114</v>
       </c>
       <c r="N3" s="44" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="O3" s="44" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="P3" s="93" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="Q3" s="61" t="n">
         <v>34604</v>
       </c>
       <c r="R3" s="44" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="S3" s="44" t="s">
         <v>119</v>
       </c>
       <c r="T3" s="44" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="V3" s="44" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="W3" s="9" t="n">
         <v>45614</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="Y3" s="93" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Z3" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AA3" s="123" t="s">
-        <v>204</v>
-      </c>
-      <c r="AB3" s="124" t="s">
+      <c r="AA3" s="124" t="s">
         <v>205</v>
+      </c>
+      <c r="AB3" s="125" t="s">
+        <v>206</v>
       </c>
       <c r="AC3" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AD3" s="125" t="n">
+      <c r="AD3" s="126" t="n">
         <v>0.548611111111111</v>
       </c>
       <c r="AE3" s="38" t="s">
         <v>132</v>
       </c>
       <c r="AF3" s="64" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AG3" s="38" t="s">
         <v>134</v>
       </c>
       <c r="AH3" s="64" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI3" s="38" t="s">
         <v>134</v>
       </c>
       <c r="AJ3" s="10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AK3" s="92" t="n">
         <v>1</v>
       </c>
       <c r="AL3" s="62" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="AM3" s="9" t="n">
         <v>45612</v>
@@ -18605,7 +18625,7 @@
         <v>177</v>
       </c>
       <c r="AP3" s="10" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="AQ3" s="10" t="s">
         <v>137</v>
@@ -18655,7 +18675,7 @@
       <c r="BK3" s="9" t="n">
         <v>45614</v>
       </c>
-      <c r="BL3" s="126" t="n">
+      <c r="BL3" s="127" t="n">
         <v>0.416666666666667</v>
       </c>
       <c r="BM3" s="62" t="s">
@@ -18673,7 +18693,7 @@
       <c r="BQ3" s="63" t="n">
         <v>45614</v>
       </c>
-      <c r="BR3" s="126" t="n">
+      <c r="BR3" s="127" t="n">
         <v>0.506944444444444</v>
       </c>
       <c r="BS3" s="63" t="s">
@@ -18695,10 +18715,10 @@
         <v>0.0701388888888889</v>
       </c>
       <c r="BY3" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="BZ3" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="CA3" s="113" t="n">
         <v>45612</v>
@@ -18707,10 +18727,10 @@
         <v>45613</v>
       </c>
       <c r="CC3" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="CD3" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="CE3" s="113" t="n">
         <v>45612</v>
@@ -18719,7 +18739,7 @@
         <v>45613</v>
       </c>
       <c r="CG3" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18740,11 +18760,11 @@
       <c r="W4" s="5"/>
       <c r="Y4" s="93"/>
       <c r="Z4" s="9"/>
-      <c r="AA4" s="123"/>
-      <c r="AB4" s="124"/>
+      <c r="AA4" s="124"/>
+      <c r="AB4" s="125"/>
       <c r="AC4" s="9"/>
-      <c r="AD4" s="125"/>
-      <c r="AE4" s="123"/>
+      <c r="AD4" s="126"/>
+      <c r="AE4" s="124"/>
       <c r="AF4" s="64"/>
       <c r="AH4" s="64"/>
       <c r="AK4" s="92"/>
@@ -18766,13 +18786,13 @@
       <c r="BI4" s="62"/>
       <c r="BJ4" s="62"/>
       <c r="BK4" s="9"/>
-      <c r="BL4" s="126"/>
+      <c r="BL4" s="127"/>
       <c r="BM4" s="62"/>
       <c r="BN4" s="63"/>
       <c r="BO4" s="62"/>
       <c r="BP4" s="62"/>
       <c r="BQ4" s="63"/>
-      <c r="BR4" s="126"/>
+      <c r="BR4" s="127"/>
       <c r="BS4" s="63"/>
       <c r="BT4" s="63"/>
       <c r="BU4" s="63"/>
@@ -18798,10 +18818,10 @@
       <c r="W5" s="9"/>
       <c r="Y5" s="93"/>
       <c r="Z5" s="9"/>
-      <c r="AA5" s="123"/>
-      <c r="AB5" s="124"/>
+      <c r="AA5" s="124"/>
+      <c r="AB5" s="125"/>
       <c r="AC5" s="9"/>
-      <c r="AD5" s="125"/>
+      <c r="AD5" s="126"/>
       <c r="AE5" s="38"/>
       <c r="AF5" s="64"/>
       <c r="AG5" s="38"/>
@@ -18826,13 +18846,13 @@
       <c r="BI5" s="62"/>
       <c r="BJ5" s="62"/>
       <c r="BK5" s="9"/>
-      <c r="BL5" s="126"/>
+      <c r="BL5" s="127"/>
       <c r="BM5" s="62"/>
       <c r="BN5" s="63"/>
       <c r="BO5" s="62"/>
       <c r="BP5" s="62"/>
       <c r="BQ5" s="63"/>
-      <c r="BR5" s="126"/>
+      <c r="BR5" s="127"/>
       <c r="BS5" s="63"/>
       <c r="BT5" s="63"/>
       <c r="BU5" s="63"/>
@@ -18858,10 +18878,10 @@
       <c r="W6" s="9"/>
       <c r="Y6" s="93"/>
       <c r="Z6" s="9"/>
-      <c r="AA6" s="123"/>
-      <c r="AB6" s="124"/>
+      <c r="AA6" s="124"/>
+      <c r="AB6" s="125"/>
       <c r="AC6" s="9"/>
-      <c r="AD6" s="125"/>
+      <c r="AD6" s="126"/>
       <c r="AE6" s="38"/>
       <c r="AF6" s="64"/>
       <c r="AG6" s="38"/>
@@ -18886,13 +18906,13 @@
       <c r="BI6" s="62"/>
       <c r="BJ6" s="62"/>
       <c r="BK6" s="9"/>
-      <c r="BL6" s="126"/>
+      <c r="BL6" s="127"/>
       <c r="BM6" s="62"/>
       <c r="BN6" s="63"/>
       <c r="BO6" s="62"/>
       <c r="BP6" s="62"/>
       <c r="BQ6" s="63"/>
-      <c r="BR6" s="126"/>
+      <c r="BR6" s="127"/>
       <c r="BS6" s="63"/>
       <c r="BT6" s="63"/>
       <c r="BU6" s="63"/>
@@ -18918,10 +18938,10 @@
       <c r="W7" s="9"/>
       <c r="Y7" s="93"/>
       <c r="Z7" s="9"/>
-      <c r="AA7" s="123"/>
-      <c r="AB7" s="124"/>
+      <c r="AA7" s="124"/>
+      <c r="AB7" s="125"/>
       <c r="AC7" s="9"/>
-      <c r="AD7" s="125"/>
+      <c r="AD7" s="126"/>
       <c r="AE7" s="38"/>
       <c r="AF7" s="64"/>
       <c r="AG7" s="38"/>
@@ -18946,13 +18966,13 @@
       <c r="BI7" s="62"/>
       <c r="BJ7" s="62"/>
       <c r="BK7" s="9"/>
-      <c r="BL7" s="126"/>
+      <c r="BL7" s="127"/>
       <c r="BM7" s="62"/>
       <c r="BN7" s="63"/>
       <c r="BO7" s="62"/>
       <c r="BP7" s="62"/>
       <c r="BQ7" s="63"/>
-      <c r="BR7" s="126"/>
+      <c r="BR7" s="127"/>
       <c r="BS7" s="63"/>
       <c r="BT7" s="63"/>
       <c r="BU7" s="63"/>
@@ -18979,10 +18999,10 @@
       <c r="W8" s="9"/>
       <c r="Y8" s="93"/>
       <c r="Z8" s="9"/>
-      <c r="AA8" s="123"/>
-      <c r="AB8" s="124"/>
+      <c r="AA8" s="124"/>
+      <c r="AB8" s="125"/>
       <c r="AC8" s="9"/>
-      <c r="AD8" s="125"/>
+      <c r="AD8" s="126"/>
       <c r="AE8" s="38"/>
       <c r="AF8" s="64"/>
       <c r="AG8" s="38"/>
@@ -19007,13 +19027,13 @@
       <c r="BI8" s="62"/>
       <c r="BJ8" s="62"/>
       <c r="BK8" s="9"/>
-      <c r="BL8" s="126"/>
+      <c r="BL8" s="127"/>
       <c r="BM8" s="62"/>
       <c r="BN8" s="63"/>
       <c r="BO8" s="62"/>
       <c r="BP8" s="62"/>
       <c r="BQ8" s="63"/>
-      <c r="BR8" s="126"/>
+      <c r="BR8" s="127"/>
       <c r="BS8" s="63"/>
       <c r="BT8" s="63"/>
       <c r="BU8" s="63"/>
@@ -19039,10 +19059,10 @@
       <c r="W9" s="9"/>
       <c r="Y9" s="93"/>
       <c r="Z9" s="9"/>
-      <c r="AA9" s="123"/>
-      <c r="AB9" s="124"/>
+      <c r="AA9" s="124"/>
+      <c r="AB9" s="125"/>
       <c r="AC9" s="9"/>
-      <c r="AD9" s="125"/>
+      <c r="AD9" s="126"/>
       <c r="AE9" s="38"/>
       <c r="AF9" s="64"/>
       <c r="AG9" s="38"/>
@@ -19067,13 +19087,13 @@
       <c r="BI9" s="62"/>
       <c r="BJ9" s="62"/>
       <c r="BK9" s="9"/>
-      <c r="BL9" s="126"/>
+      <c r="BL9" s="127"/>
       <c r="BM9" s="62"/>
       <c r="BN9" s="63"/>
       <c r="BO9" s="62"/>
       <c r="BP9" s="62"/>
       <c r="BQ9" s="63"/>
-      <c r="BR9" s="126"/>
+      <c r="BR9" s="127"/>
       <c r="BS9" s="63"/>
       <c r="BT9" s="63"/>
       <c r="BU9" s="63"/>
@@ -19099,10 +19119,10 @@
       <c r="W10" s="9"/>
       <c r="Y10" s="93"/>
       <c r="Z10" s="9"/>
-      <c r="AA10" s="123"/>
-      <c r="AB10" s="124"/>
+      <c r="AA10" s="124"/>
+      <c r="AB10" s="125"/>
       <c r="AC10" s="9"/>
-      <c r="AD10" s="125"/>
+      <c r="AD10" s="126"/>
       <c r="AE10" s="38"/>
       <c r="AF10" s="64"/>
       <c r="AG10" s="38"/>
@@ -19127,13 +19147,13 @@
       <c r="BI10" s="62"/>
       <c r="BJ10" s="62"/>
       <c r="BK10" s="9"/>
-      <c r="BL10" s="126"/>
+      <c r="BL10" s="127"/>
       <c r="BM10" s="62"/>
       <c r="BN10" s="63"/>
       <c r="BO10" s="62"/>
       <c r="BP10" s="62"/>
       <c r="BQ10" s="63"/>
-      <c r="BR10" s="126"/>
+      <c r="BR10" s="127"/>
       <c r="BS10" s="63"/>
       <c r="BT10" s="63"/>
       <c r="BU10" s="63"/>
@@ -19161,7 +19181,7 @@
       <c r="Z11" s="9"/>
       <c r="AB11" s="44"/>
       <c r="AC11" s="9"/>
-      <c r="AD11" s="125"/>
+      <c r="AD11" s="126"/>
       <c r="AE11" s="38"/>
       <c r="AF11" s="64"/>
       <c r="AG11" s="38"/>
@@ -19185,13 +19205,13 @@
       <c r="BI11" s="62"/>
       <c r="BJ11" s="62"/>
       <c r="BK11" s="9"/>
-      <c r="BL11" s="126"/>
+      <c r="BL11" s="127"/>
       <c r="BM11" s="62"/>
       <c r="BN11" s="63"/>
       <c r="BO11" s="62"/>
       <c r="BP11" s="62"/>
       <c r="BQ11" s="63"/>
-      <c r="BR11" s="126"/>
+      <c r="BR11" s="127"/>
       <c r="BS11" s="63"/>
       <c r="BT11" s="63"/>
       <c r="BU11" s="63"/>
@@ -19219,7 +19239,7 @@
       <c r="Z12" s="9"/>
       <c r="AB12" s="44"/>
       <c r="AC12" s="9"/>
-      <c r="AD12" s="125"/>
+      <c r="AD12" s="126"/>
       <c r="AE12" s="38"/>
       <c r="AF12" s="64"/>
       <c r="AG12" s="38"/>
@@ -19245,7 +19265,7 @@
       <c r="BO12" s="62"/>
       <c r="BP12" s="62"/>
       <c r="BQ12" s="63"/>
-      <c r="BR12" s="126"/>
+      <c r="BR12" s="127"/>
       <c r="BS12" s="63"/>
       <c r="BT12" s="63"/>
       <c r="BU12" s="63"/>
@@ -19273,7 +19293,7 @@
       <c r="Z13" s="9"/>
       <c r="AB13" s="44"/>
       <c r="AC13" s="9"/>
-      <c r="AD13" s="125"/>
+      <c r="AD13" s="126"/>
       <c r="AE13" s="38"/>
       <c r="AF13" s="64"/>
       <c r="AG13" s="38"/>
@@ -19295,7 +19315,7 @@
       <c r="BO13" s="62"/>
       <c r="BP13" s="62"/>
       <c r="BQ13" s="63"/>
-      <c r="BR13" s="126"/>
+      <c r="BR13" s="127"/>
       <c r="BS13" s="63"/>
       <c r="BT13" s="63"/>
       <c r="BU13" s="63"/>
@@ -19323,7 +19343,7 @@
       <c r="Z14" s="9"/>
       <c r="AB14" s="44"/>
       <c r="AC14" s="9"/>
-      <c r="AD14" s="125"/>
+      <c r="AD14" s="126"/>
       <c r="AE14" s="38"/>
       <c r="AF14" s="64"/>
       <c r="AG14" s="38"/>
@@ -19345,7 +19365,7 @@
       <c r="BO14" s="62"/>
       <c r="BP14" s="62"/>
       <c r="BQ14" s="63"/>
-      <c r="BR14" s="126"/>
+      <c r="BR14" s="127"/>
       <c r="BS14" s="63"/>
       <c r="BT14" s="63"/>
       <c r="BU14" s="63"/>
@@ -19373,7 +19393,7 @@
       <c r="Z15" s="9"/>
       <c r="AB15" s="44"/>
       <c r="AC15" s="9"/>
-      <c r="AD15" s="125"/>
+      <c r="AD15" s="126"/>
       <c r="AE15" s="38"/>
       <c r="AF15" s="64"/>
       <c r="AG15" s="38"/>
@@ -19395,7 +19415,7 @@
       <c r="BO15" s="62"/>
       <c r="BP15" s="62"/>
       <c r="BQ15" s="63"/>
-      <c r="BR15" s="126"/>
+      <c r="BR15" s="127"/>
       <c r="BS15" s="63"/>
       <c r="BT15" s="63"/>
       <c r="BU15" s="63"/>
@@ -19423,7 +19443,7 @@
       <c r="Z16" s="9"/>
       <c r="AB16" s="44"/>
       <c r="AC16" s="9"/>
-      <c r="AD16" s="125"/>
+      <c r="AD16" s="126"/>
       <c r="AE16" s="38"/>
       <c r="AF16" s="64"/>
       <c r="AG16" s="38"/>
@@ -19445,7 +19465,7 @@
       <c r="BO16" s="62"/>
       <c r="BP16" s="62"/>
       <c r="BQ16" s="63"/>
-      <c r="BR16" s="126"/>
+      <c r="BR16" s="127"/>
       <c r="BS16" s="63"/>
       <c r="BT16" s="63"/>
       <c r="BU16" s="63"/>
@@ -19473,7 +19493,7 @@
       <c r="Z17" s="9"/>
       <c r="AB17" s="44"/>
       <c r="AC17" s="9"/>
-      <c r="AD17" s="125"/>
+      <c r="AD17" s="126"/>
       <c r="AE17" s="38"/>
       <c r="AF17" s="64"/>
       <c r="AG17" s="38"/>
@@ -19495,7 +19515,7 @@
       <c r="BO17" s="62"/>
       <c r="BP17" s="62"/>
       <c r="BQ17" s="63"/>
-      <c r="BR17" s="126"/>
+      <c r="BR17" s="127"/>
       <c r="BS17" s="63"/>
       <c r="BT17" s="63"/>
       <c r="BU17" s="63"/>
@@ -19523,7 +19543,7 @@
       <c r="Z18" s="9"/>
       <c r="AB18" s="44"/>
       <c r="AC18" s="9"/>
-      <c r="AD18" s="125"/>
+      <c r="AD18" s="126"/>
       <c r="AE18" s="38"/>
       <c r="AF18" s="64"/>
       <c r="AG18" s="38"/>
@@ -19543,7 +19563,7 @@
       <c r="BO18" s="62"/>
       <c r="BP18" s="62"/>
       <c r="BQ18" s="63"/>
-      <c r="BR18" s="126"/>
+      <c r="BR18" s="127"/>
       <c r="BS18" s="63"/>
       <c r="BT18" s="63"/>
       <c r="BU18" s="63"/>
@@ -19571,7 +19591,7 @@
       <c r="Z19" s="9"/>
       <c r="AB19" s="44"/>
       <c r="AC19" s="9"/>
-      <c r="AD19" s="125"/>
+      <c r="AD19" s="126"/>
       <c r="AE19" s="38"/>
       <c r="AF19" s="64"/>
       <c r="AG19" s="38"/>
@@ -19591,7 +19611,7 @@
       <c r="BO19" s="62"/>
       <c r="BP19" s="62"/>
       <c r="BQ19" s="63"/>
-      <c r="BR19" s="126"/>
+      <c r="BR19" s="127"/>
       <c r="BS19" s="63"/>
       <c r="BT19" s="63"/>
       <c r="BU19" s="63"/>
@@ -19619,7 +19639,7 @@
       <c r="Z20" s="9"/>
       <c r="AB20" s="44"/>
       <c r="AC20" s="9"/>
-      <c r="AD20" s="125"/>
+      <c r="AD20" s="126"/>
       <c r="AE20" s="38"/>
       <c r="AF20" s="64"/>
       <c r="AG20" s="38"/>
@@ -19639,7 +19659,7 @@
       <c r="BO20" s="62"/>
       <c r="BP20" s="62"/>
       <c r="BQ20" s="63"/>
-      <c r="BR20" s="126"/>
+      <c r="BR20" s="127"/>
       <c r="BS20" s="63"/>
       <c r="BT20" s="63"/>
       <c r="BU20" s="63"/>
@@ -19667,7 +19687,7 @@
       <c r="Z21" s="9"/>
       <c r="AB21" s="44"/>
       <c r="AC21" s="9"/>
-      <c r="AD21" s="125"/>
+      <c r="AD21" s="126"/>
       <c r="AE21" s="38"/>
       <c r="AF21" s="64"/>
       <c r="AG21" s="38"/>
@@ -19685,13 +19705,13 @@
       <c r="BI21" s="62"/>
       <c r="BJ21" s="62"/>
       <c r="BK21" s="9"/>
-      <c r="BL21" s="126"/>
+      <c r="BL21" s="127"/>
       <c r="BM21" s="62"/>
       <c r="BN21" s="63"/>
       <c r="BO21" s="62"/>
       <c r="BP21" s="62"/>
       <c r="BQ21" s="63"/>
-      <c r="BR21" s="126"/>
+      <c r="BR21" s="127"/>
       <c r="BS21" s="63"/>
       <c r="BT21" s="63"/>
       <c r="BU21" s="63"/>
@@ -19719,7 +19739,7 @@
       <c r="Z22" s="9"/>
       <c r="AB22" s="44"/>
       <c r="AC22" s="9"/>
-      <c r="AD22" s="125"/>
+      <c r="AD22" s="126"/>
       <c r="AE22" s="38"/>
       <c r="AF22" s="64"/>
       <c r="AG22" s="38"/>
@@ -19740,13 +19760,13 @@
       <c r="BI22" s="62"/>
       <c r="BJ22" s="62"/>
       <c r="BK22" s="9"/>
-      <c r="BL22" s="126"/>
+      <c r="BL22" s="127"/>
       <c r="BM22" s="62"/>
       <c r="BN22" s="63"/>
       <c r="BO22" s="62"/>
       <c r="BP22" s="62"/>
       <c r="BQ22" s="63"/>
-      <c r="BR22" s="126"/>
+      <c r="BR22" s="127"/>
       <c r="BS22" s="63"/>
       <c r="BT22" s="63"/>
       <c r="BU22" s="63"/>
@@ -19774,7 +19794,7 @@
       <c r="Z23" s="9"/>
       <c r="AB23" s="44"/>
       <c r="AC23" s="9"/>
-      <c r="AD23" s="125"/>
+      <c r="AD23" s="126"/>
       <c r="AE23" s="38"/>
       <c r="AF23" s="64"/>
       <c r="AG23" s="38"/>
@@ -19796,13 +19816,13 @@
       <c r="BI23" s="62"/>
       <c r="BJ23" s="62"/>
       <c r="BK23" s="9"/>
-      <c r="BL23" s="126"/>
+      <c r="BL23" s="127"/>
       <c r="BM23" s="62"/>
       <c r="BN23" s="63"/>
       <c r="BO23" s="62"/>
       <c r="BP23" s="62"/>
       <c r="BQ23" s="63"/>
-      <c r="BR23" s="126"/>
+      <c r="BR23" s="127"/>
       <c r="BS23" s="63"/>
       <c r="BT23" s="63"/>
       <c r="BU23" s="63"/>
@@ -19830,7 +19850,7 @@
       <c r="Z24" s="9"/>
       <c r="AB24" s="44"/>
       <c r="AC24" s="9"/>
-      <c r="AD24" s="125"/>
+      <c r="AD24" s="126"/>
       <c r="AE24" s="38"/>
       <c r="AF24" s="64"/>
       <c r="AG24" s="38"/>
@@ -19852,13 +19872,13 @@
       <c r="BI24" s="62"/>
       <c r="BJ24" s="62"/>
       <c r="BK24" s="9"/>
-      <c r="BL24" s="126"/>
+      <c r="BL24" s="127"/>
       <c r="BM24" s="62"/>
       <c r="BN24" s="63"/>
       <c r="BO24" s="62"/>
       <c r="BP24" s="62"/>
       <c r="BQ24" s="63"/>
-      <c r="BR24" s="126"/>
+      <c r="BR24" s="127"/>
       <c r="BS24" s="63"/>
       <c r="BT24" s="63"/>
       <c r="BU24" s="63"/>
@@ -19886,7 +19906,7 @@
       <c r="Z25" s="9"/>
       <c r="AB25" s="44"/>
       <c r="AC25" s="9"/>
-      <c r="AD25" s="125"/>
+      <c r="AD25" s="126"/>
       <c r="AE25" s="38"/>
       <c r="AF25" s="64"/>
       <c r="AG25" s="38"/>
@@ -19908,13 +19928,13 @@
       <c r="BI25" s="62"/>
       <c r="BJ25" s="62"/>
       <c r="BK25" s="9"/>
-      <c r="BL25" s="126"/>
+      <c r="BL25" s="127"/>
       <c r="BM25" s="62"/>
       <c r="BN25" s="63"/>
       <c r="BO25" s="62"/>
       <c r="BP25" s="62"/>
       <c r="BQ25" s="63"/>
-      <c r="BR25" s="126"/>
+      <c r="BR25" s="127"/>
       <c r="BS25" s="63"/>
       <c r="BT25" s="63"/>
       <c r="BU25" s="63"/>
@@ -19942,7 +19962,7 @@
       <c r="Z26" s="9"/>
       <c r="AB26" s="44"/>
       <c r="AC26" s="9"/>
-      <c r="AD26" s="125"/>
+      <c r="AD26" s="126"/>
       <c r="AE26" s="38"/>
       <c r="AF26" s="64"/>
       <c r="AG26" s="38"/>
@@ -19964,13 +19984,13 @@
       <c r="BI26" s="62"/>
       <c r="BJ26" s="62"/>
       <c r="BK26" s="9"/>
-      <c r="BL26" s="126"/>
+      <c r="BL26" s="127"/>
       <c r="BM26" s="62"/>
       <c r="BN26" s="63"/>
       <c r="BO26" s="62"/>
       <c r="BP26" s="62"/>
       <c r="BQ26" s="63"/>
-      <c r="BR26" s="126"/>
+      <c r="BR26" s="127"/>
       <c r="BS26" s="63"/>
       <c r="BT26" s="63"/>
       <c r="BU26" s="63"/>
@@ -19998,7 +20018,7 @@
       <c r="Z27" s="9"/>
       <c r="AB27" s="44"/>
       <c r="AC27" s="9"/>
-      <c r="AD27" s="125"/>
+      <c r="AD27" s="126"/>
       <c r="AE27" s="38"/>
       <c r="AF27" s="64"/>
       <c r="AG27" s="38"/>
@@ -20020,13 +20040,13 @@
       <c r="BI27" s="62"/>
       <c r="BJ27" s="62"/>
       <c r="BK27" s="9"/>
-      <c r="BL27" s="126"/>
+      <c r="BL27" s="127"/>
       <c r="BM27" s="62"/>
       <c r="BN27" s="63"/>
       <c r="BO27" s="62"/>
       <c r="BP27" s="62"/>
       <c r="BQ27" s="63"/>
-      <c r="BR27" s="126"/>
+      <c r="BR27" s="127"/>
       <c r="BS27" s="63"/>
       <c r="BT27" s="63"/>
       <c r="BU27" s="63"/>
@@ -20054,7 +20074,7 @@
       <c r="Z28" s="9"/>
       <c r="AB28" s="44"/>
       <c r="AC28" s="9"/>
-      <c r="AD28" s="125"/>
+      <c r="AD28" s="126"/>
       <c r="AE28" s="38"/>
       <c r="AF28" s="64"/>
       <c r="AG28" s="38"/>
@@ -20076,13 +20096,13 @@
       <c r="BI28" s="62"/>
       <c r="BJ28" s="62"/>
       <c r="BK28" s="9"/>
-      <c r="BL28" s="126"/>
+      <c r="BL28" s="127"/>
       <c r="BM28" s="62"/>
       <c r="BN28" s="63"/>
       <c r="BO28" s="62"/>
       <c r="BP28" s="62"/>
       <c r="BQ28" s="63"/>
-      <c r="BR28" s="126"/>
+      <c r="BR28" s="127"/>
       <c r="BS28" s="63"/>
       <c r="BT28" s="63"/>
       <c r="BU28" s="63"/>
@@ -20110,7 +20130,7 @@
       <c r="Z29" s="9"/>
       <c r="AB29" s="44"/>
       <c r="AC29" s="9"/>
-      <c r="AD29" s="125"/>
+      <c r="AD29" s="126"/>
       <c r="AE29" s="38"/>
       <c r="AF29" s="64"/>
       <c r="AG29" s="38"/>
@@ -20132,13 +20152,13 @@
       <c r="BI29" s="62"/>
       <c r="BJ29" s="62"/>
       <c r="BK29" s="9"/>
-      <c r="BL29" s="126"/>
+      <c r="BL29" s="127"/>
       <c r="BM29" s="62"/>
       <c r="BN29" s="63"/>
       <c r="BO29" s="62"/>
       <c r="BP29" s="62"/>
       <c r="BQ29" s="63"/>
-      <c r="BR29" s="126"/>
+      <c r="BR29" s="127"/>
       <c r="BS29" s="63"/>
       <c r="BT29" s="63"/>
       <c r="BU29" s="63"/>
@@ -20166,7 +20186,7 @@
       <c r="Z30" s="9"/>
       <c r="AB30" s="44"/>
       <c r="AC30" s="9"/>
-      <c r="AD30" s="125"/>
+      <c r="AD30" s="126"/>
       <c r="AE30" s="38"/>
       <c r="AF30" s="64"/>
       <c r="AG30" s="38"/>
@@ -20188,13 +20208,13 @@
       <c r="BI30" s="62"/>
       <c r="BJ30" s="62"/>
       <c r="BK30" s="9"/>
-      <c r="BL30" s="126"/>
+      <c r="BL30" s="127"/>
       <c r="BM30" s="62"/>
       <c r="BN30" s="63"/>
       <c r="BO30" s="62"/>
       <c r="BP30" s="62"/>
       <c r="BQ30" s="63"/>
-      <c r="BR30" s="126"/>
+      <c r="BR30" s="127"/>
       <c r="BS30" s="63"/>
       <c r="BT30" s="63"/>
       <c r="BU30" s="63"/>
@@ -20222,7 +20242,7 @@
       <c r="Z31" s="9"/>
       <c r="AB31" s="44"/>
       <c r="AC31" s="9"/>
-      <c r="AD31" s="125"/>
+      <c r="AD31" s="126"/>
       <c r="AE31" s="38"/>
       <c r="AF31" s="64"/>
       <c r="AG31" s="38"/>
@@ -20244,13 +20264,13 @@
       <c r="BI31" s="62"/>
       <c r="BJ31" s="62"/>
       <c r="BK31" s="9"/>
-      <c r="BL31" s="126"/>
+      <c r="BL31" s="127"/>
       <c r="BM31" s="62"/>
       <c r="BN31" s="63"/>
       <c r="BO31" s="62"/>
       <c r="BP31" s="62"/>
       <c r="BQ31" s="63"/>
-      <c r="BR31" s="126"/>
+      <c r="BR31" s="127"/>
       <c r="BS31" s="63"/>
       <c r="BT31" s="63"/>
       <c r="BU31" s="63"/>
@@ -20258,11 +20278,11 @@
       <c r="BW31" s="63"/>
       <c r="BX31" s="68"/>
     </row>
-    <row r="32" s="128" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" s="129" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
-      <c r="D32" s="127"/>
+      <c r="D32" s="128"/>
       <c r="E32" s="61"/>
       <c r="F32" s="61"/>
       <c r="G32" s="37"/>
@@ -20287,7 +20307,7 @@
       <c r="AA32" s="44"/>
       <c r="AB32" s="44"/>
       <c r="AC32" s="9"/>
-      <c r="AD32" s="125"/>
+      <c r="AD32" s="126"/>
       <c r="AE32" s="38"/>
       <c r="AF32" s="64"/>
       <c r="AG32" s="38"/>
@@ -20299,42 +20319,42 @@
       <c r="AN32" s="9"/>
       <c r="AR32" s="9"/>
       <c r="AS32" s="9"/>
-      <c r="AW32" s="129"/>
-      <c r="AX32" s="129"/>
+      <c r="AW32" s="130"/>
+      <c r="AX32" s="130"/>
       <c r="BA32" s="69"/>
       <c r="BB32" s="69"/>
       <c r="BC32" s="69"/>
       <c r="BD32" s="69"/>
-      <c r="BE32" s="130"/>
-      <c r="BF32" s="131"/>
+      <c r="BE32" s="131"/>
+      <c r="BF32" s="132"/>
       <c r="BG32" s="69"/>
       <c r="BH32" s="69"/>
       <c r="BI32" s="69"/>
       <c r="BJ32" s="69"/>
       <c r="BK32" s="9"/>
-      <c r="BL32" s="132"/>
+      <c r="BL32" s="133"/>
       <c r="BM32" s="69"/>
-      <c r="BN32" s="130"/>
+      <c r="BN32" s="131"/>
       <c r="BO32" s="69"/>
-      <c r="BP32" s="133"/>
-      <c r="BQ32" s="130"/>
-      <c r="BR32" s="132"/>
-      <c r="BS32" s="130"/>
-      <c r="BT32" s="130"/>
-      <c r="BU32" s="130"/>
-      <c r="BV32" s="130"/>
-      <c r="BW32" s="130"/>
+      <c r="BP32" s="134"/>
+      <c r="BQ32" s="131"/>
+      <c r="BR32" s="133"/>
+      <c r="BS32" s="131"/>
+      <c r="BT32" s="131"/>
+      <c r="BU32" s="131"/>
+      <c r="BV32" s="131"/>
+      <c r="BW32" s="131"/>
       <c r="BX32" s="68"/>
       <c r="BY32" s="1"/>
-      <c r="CA32" s="129"/>
-      <c r="CB32" s="129"/>
-      <c r="CE32" s="129"/>
-      <c r="CF32" s="129"/>
-      <c r="CL32" s="133"/>
-      <c r="CM32" s="133"/>
-      <c r="CN32" s="133"/>
-      <c r="CO32" s="134"/>
-      <c r="CP32" s="133"/>
+      <c r="CA32" s="130"/>
+      <c r="CB32" s="130"/>
+      <c r="CE32" s="130"/>
+      <c r="CF32" s="130"/>
+      <c r="CL32" s="134"/>
+      <c r="CM32" s="134"/>
+      <c r="CN32" s="134"/>
+      <c r="CO32" s="135"/>
+      <c r="CP32" s="134"/>
     </row>
     <row r="33" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E33" s="61"/>
@@ -20357,7 +20377,7 @@
       <c r="Z33" s="9"/>
       <c r="AB33" s="44"/>
       <c r="AC33" s="9"/>
-      <c r="AD33" s="125"/>
+      <c r="AD33" s="126"/>
       <c r="AE33" s="38"/>
       <c r="AF33" s="64"/>
       <c r="AG33" s="38"/>
@@ -20379,12 +20399,12 @@
       <c r="BI33" s="62"/>
       <c r="BJ33" s="62"/>
       <c r="BK33" s="9"/>
-      <c r="BL33" s="126"/>
+      <c r="BL33" s="127"/>
       <c r="BM33" s="62"/>
       <c r="BN33" s="63"/>
       <c r="BO33" s="62"/>
       <c r="BQ33" s="63"/>
-      <c r="BR33" s="126"/>
+      <c r="BR33" s="127"/>
       <c r="BS33" s="63"/>
       <c r="BT33" s="63"/>
       <c r="BU33" s="63"/>
@@ -20392,11 +20412,11 @@
       <c r="BW33" s="63"/>
       <c r="BX33" s="68"/>
     </row>
-    <row r="34" s="128" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" s="129" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
-      <c r="D34" s="127"/>
+      <c r="D34" s="128"/>
       <c r="E34" s="61"/>
       <c r="F34" s="61"/>
       <c r="G34" s="37"/>
@@ -20414,59 +20434,59 @@
       <c r="S34" s="44"/>
       <c r="T34" s="44"/>
       <c r="V34" s="44"/>
-      <c r="X34" s="135"/>
+      <c r="X34" s="136"/>
       <c r="Y34" s="93"/>
-      <c r="Z34" s="136"/>
+      <c r="Z34" s="137"/>
       <c r="AB34" s="44"/>
-      <c r="AC34" s="136"/>
-      <c r="AD34" s="125"/>
-      <c r="AE34" s="137"/>
+      <c r="AC34" s="137"/>
+      <c r="AD34" s="126"/>
+      <c r="AE34" s="138"/>
       <c r="AK34" s="92"/>
-      <c r="AM34" s="129"/>
-      <c r="AN34" s="129"/>
-      <c r="AR34" s="129"/>
-      <c r="AS34" s="129"/>
-      <c r="AW34" s="129"/>
-      <c r="AX34" s="129"/>
+      <c r="AM34" s="130"/>
+      <c r="AN34" s="130"/>
+      <c r="AR34" s="130"/>
+      <c r="AS34" s="130"/>
+      <c r="AW34" s="130"/>
+      <c r="AX34" s="130"/>
       <c r="BA34" s="69"/>
       <c r="BB34" s="69"/>
       <c r="BC34" s="69"/>
       <c r="BD34" s="69"/>
-      <c r="BE34" s="130"/>
-      <c r="BF34" s="131"/>
+      <c r="BE34" s="131"/>
+      <c r="BF34" s="132"/>
       <c r="BG34" s="69"/>
       <c r="BH34" s="69"/>
       <c r="BI34" s="69"/>
       <c r="BJ34" s="69"/>
       <c r="BK34" s="5"/>
-      <c r="BL34" s="132"/>
+      <c r="BL34" s="133"/>
       <c r="BM34" s="69"/>
-      <c r="BN34" s="130"/>
+      <c r="BN34" s="131"/>
       <c r="BO34" s="69"/>
-      <c r="BQ34" s="130"/>
-      <c r="BR34" s="132"/>
-      <c r="BS34" s="130"/>
-      <c r="BT34" s="130"/>
-      <c r="BU34" s="130"/>
-      <c r="BV34" s="130"/>
-      <c r="BW34" s="130"/>
+      <c r="BQ34" s="131"/>
+      <c r="BR34" s="133"/>
+      <c r="BS34" s="131"/>
+      <c r="BT34" s="131"/>
+      <c r="BU34" s="131"/>
+      <c r="BV34" s="131"/>
+      <c r="BW34" s="131"/>
       <c r="BX34" s="68"/>
-      <c r="BY34" s="133"/>
-      <c r="CA34" s="129"/>
-      <c r="CB34" s="129"/>
-      <c r="CE34" s="129"/>
-      <c r="CF34" s="129"/>
-      <c r="CL34" s="133"/>
-      <c r="CM34" s="133"/>
-      <c r="CN34" s="133"/>
-      <c r="CO34" s="134"/>
-      <c r="CP34" s="133"/>
-    </row>
-    <row r="35" s="128" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="BY34" s="134"/>
+      <c r="CA34" s="130"/>
+      <c r="CB34" s="130"/>
+      <c r="CE34" s="130"/>
+      <c r="CF34" s="130"/>
+      <c r="CL34" s="134"/>
+      <c r="CM34" s="134"/>
+      <c r="CN34" s="134"/>
+      <c r="CO34" s="135"/>
+      <c r="CP34" s="134"/>
+    </row>
+    <row r="35" s="129" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
-      <c r="D35" s="127"/>
+      <c r="D35" s="128"/>
       <c r="E35" s="61"/>
       <c r="F35" s="61"/>
       <c r="G35" s="37"/>
@@ -20484,59 +20504,59 @@
       <c r="S35" s="44"/>
       <c r="T35" s="44"/>
       <c r="V35" s="44"/>
-      <c r="X35" s="135"/>
+      <c r="X35" s="136"/>
       <c r="Y35" s="93"/>
-      <c r="Z35" s="138"/>
+      <c r="Z35" s="139"/>
       <c r="AB35" s="44"/>
-      <c r="AC35" s="136"/>
-      <c r="AD35" s="125"/>
-      <c r="AE35" s="137"/>
+      <c r="AC35" s="137"/>
+      <c r="AD35" s="126"/>
+      <c r="AE35" s="138"/>
       <c r="AK35" s="92"/>
-      <c r="AM35" s="129"/>
-      <c r="AN35" s="129"/>
-      <c r="AR35" s="129"/>
-      <c r="AS35" s="129"/>
-      <c r="AW35" s="129"/>
-      <c r="AX35" s="129"/>
+      <c r="AM35" s="130"/>
+      <c r="AN35" s="130"/>
+      <c r="AR35" s="130"/>
+      <c r="AS35" s="130"/>
+      <c r="AW35" s="130"/>
+      <c r="AX35" s="130"/>
       <c r="BA35" s="69"/>
       <c r="BB35" s="69"/>
       <c r="BC35" s="69"/>
       <c r="BD35" s="69"/>
-      <c r="BE35" s="130"/>
-      <c r="BF35" s="131"/>
+      <c r="BE35" s="131"/>
+      <c r="BF35" s="132"/>
       <c r="BG35" s="69"/>
       <c r="BH35" s="69"/>
       <c r="BI35" s="69"/>
       <c r="BJ35" s="69"/>
-      <c r="BK35" s="139"/>
-      <c r="BL35" s="132"/>
+      <c r="BK35" s="140"/>
+      <c r="BL35" s="133"/>
       <c r="BM35" s="69"/>
-      <c r="BN35" s="130"/>
+      <c r="BN35" s="131"/>
       <c r="BO35" s="69"/>
-      <c r="BQ35" s="130"/>
-      <c r="BR35" s="132"/>
-      <c r="BS35" s="130"/>
-      <c r="BT35" s="130"/>
-      <c r="BU35" s="130"/>
-      <c r="BV35" s="130"/>
-      <c r="BW35" s="130"/>
+      <c r="BQ35" s="131"/>
+      <c r="BR35" s="133"/>
+      <c r="BS35" s="131"/>
+      <c r="BT35" s="131"/>
+      <c r="BU35" s="131"/>
+      <c r="BV35" s="131"/>
+      <c r="BW35" s="131"/>
       <c r="BX35" s="68"/>
-      <c r="BY35" s="133"/>
-      <c r="CA35" s="129"/>
-      <c r="CB35" s="129"/>
-      <c r="CE35" s="129"/>
-      <c r="CF35" s="129"/>
-      <c r="CL35" s="133"/>
-      <c r="CM35" s="133"/>
-      <c r="CN35" s="133"/>
-      <c r="CO35" s="134"/>
-      <c r="CP35" s="133"/>
-    </row>
-    <row r="36" s="128" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="BY35" s="134"/>
+      <c r="CA35" s="130"/>
+      <c r="CB35" s="130"/>
+      <c r="CE35" s="130"/>
+      <c r="CF35" s="130"/>
+      <c r="CL35" s="134"/>
+      <c r="CM35" s="134"/>
+      <c r="CN35" s="134"/>
+      <c r="CO35" s="135"/>
+      <c r="CP35" s="134"/>
+    </row>
+    <row r="36" s="129" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
-      <c r="D36" s="127"/>
+      <c r="D36" s="128"/>
       <c r="E36" s="61"/>
       <c r="F36" s="61"/>
       <c r="G36" s="37"/>
@@ -20554,60 +20574,60 @@
       <c r="S36" s="44"/>
       <c r="T36" s="44"/>
       <c r="V36" s="44"/>
-      <c r="X36" s="135"/>
+      <c r="X36" s="136"/>
       <c r="Y36" s="93"/>
-      <c r="Z36" s="138"/>
+      <c r="Z36" s="139"/>
       <c r="AB36" s="44"/>
-      <c r="AC36" s="136"/>
-      <c r="AD36" s="125"/>
-      <c r="AE36" s="137"/>
+      <c r="AC36" s="137"/>
+      <c r="AD36" s="126"/>
+      <c r="AE36" s="138"/>
       <c r="AK36" s="92"/>
-      <c r="AM36" s="129"/>
-      <c r="AN36" s="129"/>
-      <c r="AR36" s="129"/>
-      <c r="AS36" s="129"/>
-      <c r="AW36" s="129"/>
-      <c r="AX36" s="129"/>
+      <c r="AM36" s="130"/>
+      <c r="AN36" s="130"/>
+      <c r="AR36" s="130"/>
+      <c r="AS36" s="130"/>
+      <c r="AW36" s="130"/>
+      <c r="AX36" s="130"/>
       <c r="BA36" s="69"/>
       <c r="BB36" s="69"/>
       <c r="BC36" s="69"/>
       <c r="BD36" s="69"/>
-      <c r="BE36" s="130"/>
-      <c r="BF36" s="131"/>
+      <c r="BE36" s="131"/>
+      <c r="BF36" s="132"/>
       <c r="BG36" s="69"/>
       <c r="BH36" s="69"/>
       <c r="BI36" s="69"/>
       <c r="BJ36" s="69"/>
-      <c r="BK36" s="139"/>
-      <c r="BL36" s="132"/>
+      <c r="BK36" s="140"/>
+      <c r="BL36" s="133"/>
       <c r="BM36" s="69"/>
-      <c r="BN36" s="130"/>
+      <c r="BN36" s="131"/>
       <c r="BO36" s="69"/>
       <c r="BP36" s="69"/>
-      <c r="BQ36" s="130"/>
-      <c r="BR36" s="132"/>
-      <c r="BS36" s="130"/>
-      <c r="BT36" s="130"/>
-      <c r="BU36" s="130"/>
-      <c r="BV36" s="130"/>
-      <c r="BW36" s="130"/>
+      <c r="BQ36" s="131"/>
+      <c r="BR36" s="133"/>
+      <c r="BS36" s="131"/>
+      <c r="BT36" s="131"/>
+      <c r="BU36" s="131"/>
+      <c r="BV36" s="131"/>
+      <c r="BW36" s="131"/>
       <c r="BX36" s="68"/>
-      <c r="BY36" s="133"/>
-      <c r="CA36" s="129"/>
-      <c r="CB36" s="129"/>
-      <c r="CE36" s="129"/>
-      <c r="CF36" s="129"/>
-      <c r="CL36" s="133"/>
-      <c r="CM36" s="133"/>
-      <c r="CN36" s="133"/>
-      <c r="CO36" s="134"/>
-      <c r="CP36" s="133"/>
-    </row>
-    <row r="37" s="128" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="BY36" s="134"/>
+      <c r="CA36" s="130"/>
+      <c r="CB36" s="130"/>
+      <c r="CE36" s="130"/>
+      <c r="CF36" s="130"/>
+      <c r="CL36" s="134"/>
+      <c r="CM36" s="134"/>
+      <c r="CN36" s="134"/>
+      <c r="CO36" s="135"/>
+      <c r="CP36" s="134"/>
+    </row>
+    <row r="37" s="129" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
-      <c r="D37" s="127"/>
+      <c r="D37" s="128"/>
       <c r="E37" s="61"/>
       <c r="F37" s="61"/>
       <c r="G37" s="37"/>
@@ -20627,52 +20647,52 @@
       <c r="V37" s="44"/>
       <c r="X37" s="3"/>
       <c r="Y37" s="93"/>
-      <c r="Z37" s="138"/>
+      <c r="Z37" s="139"/>
       <c r="AB37" s="44"/>
-      <c r="AC37" s="136"/>
-      <c r="AD37" s="125"/>
-      <c r="AE37" s="137"/>
+      <c r="AC37" s="137"/>
+      <c r="AD37" s="126"/>
+      <c r="AE37" s="138"/>
       <c r="AK37" s="92"/>
-      <c r="AM37" s="129"/>
-      <c r="AN37" s="129"/>
-      <c r="AR37" s="129"/>
-      <c r="AS37" s="129"/>
-      <c r="AW37" s="129"/>
-      <c r="AX37" s="129"/>
+      <c r="AM37" s="130"/>
+      <c r="AN37" s="130"/>
+      <c r="AR37" s="130"/>
+      <c r="AS37" s="130"/>
+      <c r="AW37" s="130"/>
+      <c r="AX37" s="130"/>
       <c r="BA37" s="69"/>
       <c r="BB37" s="69"/>
       <c r="BC37" s="69"/>
       <c r="BD37" s="69"/>
-      <c r="BE37" s="130"/>
-      <c r="BF37" s="131"/>
+      <c r="BE37" s="131"/>
+      <c r="BF37" s="132"/>
       <c r="BG37" s="69"/>
       <c r="BH37" s="69"/>
       <c r="BI37" s="69"/>
       <c r="BJ37" s="69"/>
-      <c r="BK37" s="139"/>
-      <c r="BL37" s="132"/>
+      <c r="BK37" s="140"/>
+      <c r="BL37" s="133"/>
       <c r="BM37" s="69"/>
-      <c r="BN37" s="130"/>
+      <c r="BN37" s="131"/>
       <c r="BO37" s="69"/>
       <c r="BP37" s="69"/>
-      <c r="BQ37" s="130"/>
-      <c r="BR37" s="132"/>
-      <c r="BS37" s="130"/>
-      <c r="BT37" s="130"/>
-      <c r="BU37" s="130"/>
-      <c r="BV37" s="130"/>
-      <c r="BW37" s="130"/>
+      <c r="BQ37" s="131"/>
+      <c r="BR37" s="133"/>
+      <c r="BS37" s="131"/>
+      <c r="BT37" s="131"/>
+      <c r="BU37" s="131"/>
+      <c r="BV37" s="131"/>
+      <c r="BW37" s="131"/>
       <c r="BX37" s="68"/>
-      <c r="BY37" s="133"/>
-      <c r="CA37" s="129"/>
-      <c r="CB37" s="129"/>
-      <c r="CE37" s="129"/>
-      <c r="CF37" s="129"/>
-      <c r="CL37" s="133"/>
-      <c r="CM37" s="133"/>
-      <c r="CN37" s="133"/>
-      <c r="CO37" s="134"/>
-      <c r="CP37" s="133"/>
+      <c r="BY37" s="134"/>
+      <c r="CA37" s="130"/>
+      <c r="CB37" s="130"/>
+      <c r="CE37" s="130"/>
+      <c r="CF37" s="130"/>
+      <c r="CL37" s="134"/>
+      <c r="CM37" s="134"/>
+      <c r="CN37" s="134"/>
+      <c r="CO37" s="135"/>
+      <c r="CP37" s="134"/>
     </row>
     <row r="38" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E38" s="61"/>
@@ -20695,7 +20715,7 @@
       <c r="Y38" s="93"/>
       <c r="Z38" s="9"/>
       <c r="AB38" s="44"/>
-      <c r="AD38" s="125"/>
+      <c r="AD38" s="126"/>
       <c r="AE38" s="38"/>
       <c r="AF38" s="64"/>
       <c r="AG38" s="38"/>
@@ -20713,13 +20733,13 @@
       <c r="BI38" s="62"/>
       <c r="BJ38" s="62"/>
       <c r="BK38" s="65"/>
-      <c r="BL38" s="126"/>
+      <c r="BL38" s="127"/>
       <c r="BM38" s="62"/>
       <c r="BN38" s="63"/>
       <c r="BO38" s="62"/>
       <c r="BP38" s="62"/>
       <c r="BQ38" s="63"/>
-      <c r="BR38" s="126"/>
+      <c r="BR38" s="127"/>
       <c r="BS38" s="63"/>
       <c r="BT38" s="63"/>
       <c r="BU38" s="63"/>
@@ -20748,7 +20768,7 @@
       <c r="Y39" s="93"/>
       <c r="Z39" s="9"/>
       <c r="AB39" s="44"/>
-      <c r="AD39" s="125"/>
+      <c r="AD39" s="126"/>
       <c r="AE39" s="38"/>
       <c r="AF39" s="64"/>
       <c r="AG39" s="38"/>
@@ -20766,13 +20786,13 @@
       <c r="BI39" s="62"/>
       <c r="BJ39" s="62"/>
       <c r="BK39" s="65"/>
-      <c r="BL39" s="126"/>
+      <c r="BL39" s="127"/>
       <c r="BM39" s="62"/>
       <c r="BN39" s="63"/>
       <c r="BO39" s="62"/>
       <c r="BP39" s="62"/>
       <c r="BQ39" s="63"/>
-      <c r="BR39" s="126"/>
+      <c r="BR39" s="127"/>
       <c r="BS39" s="63"/>
       <c r="BT39" s="63"/>
       <c r="BU39" s="63"/>
@@ -20801,7 +20821,7 @@
       <c r="Y40" s="93"/>
       <c r="Z40" s="9"/>
       <c r="AB40" s="44"/>
-      <c r="AD40" s="125"/>
+      <c r="AD40" s="126"/>
       <c r="AE40" s="38"/>
       <c r="AF40" s="64"/>
       <c r="AG40" s="38"/>
@@ -20819,13 +20839,13 @@
       <c r="BI40" s="62"/>
       <c r="BJ40" s="62"/>
       <c r="BK40" s="65"/>
-      <c r="BL40" s="126"/>
+      <c r="BL40" s="127"/>
       <c r="BM40" s="62"/>
       <c r="BN40" s="63"/>
       <c r="BO40" s="62"/>
       <c r="BP40" s="62"/>
       <c r="BQ40" s="63"/>
-      <c r="BR40" s="126"/>
+      <c r="BR40" s="127"/>
       <c r="BS40" s="63"/>
       <c r="BT40" s="63"/>
       <c r="BU40" s="63"/>
@@ -20854,7 +20874,7 @@
       <c r="Y41" s="93"/>
       <c r="Z41" s="9"/>
       <c r="AB41" s="44"/>
-      <c r="AD41" s="125"/>
+      <c r="AD41" s="126"/>
       <c r="AE41" s="38"/>
       <c r="AF41" s="64"/>
       <c r="AG41" s="38"/>
@@ -20872,7 +20892,7 @@
       <c r="BI41" s="62"/>
       <c r="BJ41" s="62"/>
       <c r="BK41" s="65"/>
-      <c r="BL41" s="126"/>
+      <c r="BL41" s="127"/>
       <c r="BM41" s="62"/>
       <c r="BN41" s="63"/>
       <c r="BO41" s="62"/>
@@ -20907,7 +20927,7 @@
       <c r="Y42" s="93"/>
       <c r="Z42" s="9"/>
       <c r="AB42" s="44"/>
-      <c r="AD42" s="125"/>
+      <c r="AD42" s="126"/>
       <c r="AE42" s="38"/>
       <c r="AF42" s="64"/>
       <c r="AG42" s="38"/>
@@ -20925,7 +20945,7 @@
       <c r="BI42" s="62"/>
       <c r="BJ42" s="62"/>
       <c r="BK42" s="65"/>
-      <c r="BL42" s="126"/>
+      <c r="BL42" s="127"/>
       <c r="BM42" s="62"/>
       <c r="BN42" s="63"/>
       <c r="BO42" s="62"/>
@@ -20960,7 +20980,7 @@
       <c r="Y43" s="93"/>
       <c r="Z43" s="9"/>
       <c r="AB43" s="44"/>
-      <c r="AD43" s="125"/>
+      <c r="AD43" s="126"/>
       <c r="AE43" s="38"/>
       <c r="AF43" s="64"/>
       <c r="AG43" s="38"/>
@@ -20978,7 +20998,7 @@
       <c r="BI43" s="62"/>
       <c r="BJ43" s="62"/>
       <c r="BK43" s="65"/>
-      <c r="BL43" s="126"/>
+      <c r="BL43" s="127"/>
       <c r="BM43" s="62"/>
       <c r="BN43" s="63"/>
       <c r="BO43" s="62"/>
@@ -21013,7 +21033,7 @@
       <c r="Y44" s="93"/>
       <c r="Z44" s="9"/>
       <c r="AB44" s="44"/>
-      <c r="AD44" s="125"/>
+      <c r="AD44" s="126"/>
       <c r="AE44" s="38"/>
       <c r="AF44" s="64"/>
       <c r="AG44" s="38"/>
@@ -21031,7 +21051,7 @@
       <c r="BI44" s="62"/>
       <c r="BJ44" s="62"/>
       <c r="BK44" s="65"/>
-      <c r="BL44" s="126"/>
+      <c r="BL44" s="127"/>
       <c r="BM44" s="62"/>
       <c r="BN44" s="63"/>
       <c r="BO44" s="62"/>
@@ -21066,7 +21086,7 @@
       <c r="Y45" s="93"/>
       <c r="Z45" s="9"/>
       <c r="AB45" s="44"/>
-      <c r="AD45" s="125"/>
+      <c r="AD45" s="126"/>
       <c r="AE45" s="38"/>
       <c r="AF45" s="64"/>
       <c r="AG45" s="38"/>
@@ -21084,7 +21104,7 @@
       <c r="BI45" s="62"/>
       <c r="BJ45" s="62"/>
       <c r="BK45" s="65"/>
-      <c r="BL45" s="126"/>
+      <c r="BL45" s="127"/>
       <c r="BM45" s="62"/>
       <c r="BN45" s="63"/>
       <c r="BO45" s="62"/>
@@ -21119,7 +21139,7 @@
       <c r="Y46" s="93"/>
       <c r="Z46" s="9"/>
       <c r="AB46" s="44"/>
-      <c r="AD46" s="125"/>
+      <c r="AD46" s="126"/>
       <c r="AE46" s="38"/>
       <c r="AF46" s="64"/>
       <c r="AG46" s="38"/>
@@ -21137,7 +21157,7 @@
       <c r="BI46" s="62"/>
       <c r="BJ46" s="62"/>
       <c r="BK46" s="65"/>
-      <c r="BL46" s="126"/>
+      <c r="BL46" s="127"/>
       <c r="BM46" s="62"/>
       <c r="BN46" s="63"/>
       <c r="BO46" s="62"/>
@@ -21172,7 +21192,7 @@
       <c r="Y47" s="93"/>
       <c r="Z47" s="9"/>
       <c r="AB47" s="44"/>
-      <c r="AD47" s="125"/>
+      <c r="AD47" s="126"/>
       <c r="AE47" s="38"/>
       <c r="AF47" s="64"/>
       <c r="AG47" s="38"/>
@@ -21190,7 +21210,7 @@
       <c r="BI47" s="62"/>
       <c r="BJ47" s="62"/>
       <c r="BK47" s="65"/>
-      <c r="BL47" s="126"/>
+      <c r="BL47" s="127"/>
       <c r="BM47" s="62"/>
       <c r="BN47" s="63"/>
       <c r="BO47" s="62"/>
@@ -21225,7 +21245,7 @@
       <c r="Y48" s="93"/>
       <c r="Z48" s="9"/>
       <c r="AB48" s="44"/>
-      <c r="AD48" s="125"/>
+      <c r="AD48" s="126"/>
       <c r="AE48" s="38"/>
       <c r="AF48" s="64"/>
       <c r="AG48" s="38"/>
@@ -21243,7 +21263,7 @@
       <c r="BI48" s="62"/>
       <c r="BJ48" s="62"/>
       <c r="BK48" s="65"/>
-      <c r="BL48" s="126"/>
+      <c r="BL48" s="127"/>
       <c r="BM48" s="62"/>
       <c r="BN48" s="63"/>
       <c r="BO48" s="62"/>
@@ -21277,7 +21297,7 @@
       <c r="Y49" s="93"/>
       <c r="Z49" s="9"/>
       <c r="AB49" s="44"/>
-      <c r="AD49" s="125"/>
+      <c r="AD49" s="126"/>
       <c r="AE49" s="38"/>
       <c r="AF49" s="64"/>
       <c r="AG49" s="38"/>
@@ -21295,7 +21315,7 @@
       <c r="BI49" s="62"/>
       <c r="BJ49" s="62"/>
       <c r="BK49" s="65"/>
-      <c r="BL49" s="126"/>
+      <c r="BL49" s="127"/>
       <c r="BM49" s="62"/>
       <c r="BN49" s="63"/>
       <c r="BO49" s="62"/>
@@ -21329,7 +21349,7 @@
       <c r="Y50" s="93"/>
       <c r="Z50" s="9"/>
       <c r="AB50" s="44"/>
-      <c r="AD50" s="125"/>
+      <c r="AD50" s="126"/>
       <c r="AE50" s="38"/>
       <c r="AF50" s="64"/>
       <c r="AG50" s="38"/>
@@ -21347,7 +21367,7 @@
       <c r="BI50" s="62"/>
       <c r="BJ50" s="62"/>
       <c r="BK50" s="65"/>
-      <c r="BL50" s="126"/>
+      <c r="BL50" s="127"/>
       <c r="BM50" s="62"/>
       <c r="BN50" s="63"/>
       <c r="BO50" s="62"/>
@@ -21381,7 +21401,7 @@
       <c r="Y51" s="93"/>
       <c r="Z51" s="9"/>
       <c r="AB51" s="44"/>
-      <c r="AD51" s="125"/>
+      <c r="AD51" s="126"/>
       <c r="AE51" s="38"/>
       <c r="AF51" s="64"/>
       <c r="AG51" s="38"/>
@@ -21399,7 +21419,7 @@
       <c r="BI51" s="62"/>
       <c r="BJ51" s="62"/>
       <c r="BK51" s="65"/>
-      <c r="BL51" s="126"/>
+      <c r="BL51" s="127"/>
       <c r="BM51" s="62"/>
       <c r="BN51" s="63"/>
       <c r="BO51" s="62"/>
@@ -21433,7 +21453,7 @@
       <c r="Y52" s="93"/>
       <c r="Z52" s="9"/>
       <c r="AB52" s="44"/>
-      <c r="AD52" s="125"/>
+      <c r="AD52" s="126"/>
       <c r="AE52" s="38"/>
       <c r="AF52" s="64"/>
       <c r="AG52" s="38"/>
@@ -21451,7 +21471,7 @@
       <c r="BI52" s="62"/>
       <c r="BJ52" s="62"/>
       <c r="BK52" s="65"/>
-      <c r="BL52" s="126"/>
+      <c r="BL52" s="127"/>
       <c r="BM52" s="62"/>
       <c r="BN52" s="63"/>
       <c r="BO52" s="62"/>
@@ -21485,7 +21505,7 @@
       <c r="Y53" s="93"/>
       <c r="Z53" s="9"/>
       <c r="AB53" s="44"/>
-      <c r="AD53" s="125"/>
+      <c r="AD53" s="126"/>
       <c r="AE53" s="38"/>
       <c r="AF53" s="64"/>
       <c r="AG53" s="38"/>
@@ -21503,7 +21523,7 @@
       <c r="BI53" s="62"/>
       <c r="BJ53" s="62"/>
       <c r="BK53" s="65"/>
-      <c r="BL53" s="126"/>
+      <c r="BL53" s="127"/>
       <c r="BM53" s="62"/>
       <c r="BN53" s="63"/>
       <c r="BO53" s="62"/>
@@ -21537,7 +21557,7 @@
       <c r="Y54" s="93"/>
       <c r="Z54" s="9"/>
       <c r="AB54" s="44"/>
-      <c r="AD54" s="125"/>
+      <c r="AD54" s="126"/>
       <c r="AE54" s="38"/>
       <c r="AF54" s="64"/>
       <c r="AG54" s="38"/>
@@ -21555,7 +21575,7 @@
       <c r="BI54" s="62"/>
       <c r="BJ54" s="62"/>
       <c r="BK54" s="65"/>
-      <c r="BL54" s="126"/>
+      <c r="BL54" s="127"/>
       <c r="BM54" s="62"/>
       <c r="BN54" s="63"/>
       <c r="BO54" s="62"/>
@@ -21589,7 +21609,7 @@
       <c r="Y55" s="93"/>
       <c r="Z55" s="9"/>
       <c r="AB55" s="44"/>
-      <c r="AD55" s="125"/>
+      <c r="AD55" s="126"/>
       <c r="AE55" s="38"/>
       <c r="AF55" s="64"/>
       <c r="AG55" s="38"/>
@@ -21607,7 +21627,7 @@
       <c r="BI55" s="62"/>
       <c r="BJ55" s="62"/>
       <c r="BK55" s="65"/>
-      <c r="BL55" s="126"/>
+      <c r="BL55" s="127"/>
       <c r="BM55" s="62"/>
       <c r="BN55" s="63"/>
       <c r="BO55" s="62"/>
@@ -21641,7 +21661,7 @@
       <c r="Y56" s="93"/>
       <c r="Z56" s="9"/>
       <c r="AB56" s="44"/>
-      <c r="AD56" s="125"/>
+      <c r="AD56" s="126"/>
       <c r="AE56" s="38"/>
       <c r="AF56" s="64"/>
       <c r="AG56" s="38"/>
@@ -21659,7 +21679,7 @@
       <c r="BI56" s="62"/>
       <c r="BJ56" s="62"/>
       <c r="BK56" s="65"/>
-      <c r="BL56" s="126"/>
+      <c r="BL56" s="127"/>
       <c r="BM56" s="62"/>
       <c r="BN56" s="63"/>
       <c r="BO56" s="62"/>
@@ -21670,7 +21690,7 @@
       <c r="BU56" s="63"/>
       <c r="BV56" s="63"/>
       <c r="BW56" s="63"/>
-      <c r="BX56" s="126"/>
+      <c r="BX56" s="127"/>
     </row>
     <row r="57" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E57" s="61"/>
@@ -21693,7 +21713,7 @@
       <c r="Y57" s="93"/>
       <c r="Z57" s="9"/>
       <c r="AB57" s="44"/>
-      <c r="AD57" s="125"/>
+      <c r="AD57" s="126"/>
       <c r="AE57" s="38"/>
       <c r="AF57" s="64"/>
       <c r="AG57" s="38"/>
@@ -21711,7 +21731,7 @@
       <c r="BI57" s="62"/>
       <c r="BJ57" s="62"/>
       <c r="BK57" s="65"/>
-      <c r="BL57" s="126"/>
+      <c r="BL57" s="127"/>
       <c r="BM57" s="62"/>
       <c r="BN57" s="63"/>
       <c r="BO57" s="62"/>
@@ -21722,7 +21742,7 @@
       <c r="BU57" s="63"/>
       <c r="BV57" s="63"/>
       <c r="BW57" s="63"/>
-      <c r="BX57" s="126"/>
+      <c r="BX57" s="127"/>
     </row>
     <row r="58" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E58" s="61"/>
@@ -21745,7 +21765,7 @@
       <c r="Y58" s="93"/>
       <c r="Z58" s="9"/>
       <c r="AB58" s="44"/>
-      <c r="AD58" s="125"/>
+      <c r="AD58" s="126"/>
       <c r="AE58" s="38"/>
       <c r="AF58" s="64"/>
       <c r="AG58" s="38"/>
@@ -21763,7 +21783,7 @@
       <c r="BI58" s="62"/>
       <c r="BJ58" s="62"/>
       <c r="BK58" s="65"/>
-      <c r="BL58" s="126"/>
+      <c r="BL58" s="127"/>
       <c r="BM58" s="62"/>
       <c r="BN58" s="63"/>
       <c r="BO58" s="62"/>
@@ -21774,7 +21794,7 @@
       <c r="BU58" s="63"/>
       <c r="BV58" s="63"/>
       <c r="BW58" s="63"/>
-      <c r="BX58" s="126"/>
+      <c r="BX58" s="127"/>
     </row>
     <row r="59" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E59" s="61"/>
@@ -21797,7 +21817,7 @@
       <c r="Y59" s="93"/>
       <c r="Z59" s="9"/>
       <c r="AB59" s="44"/>
-      <c r="AD59" s="125"/>
+      <c r="AD59" s="126"/>
       <c r="AE59" s="38"/>
       <c r="AF59" s="64"/>
       <c r="AG59" s="38"/>
@@ -21815,7 +21835,7 @@
       <c r="BI59" s="62"/>
       <c r="BJ59" s="62"/>
       <c r="BK59" s="63"/>
-      <c r="BL59" s="126"/>
+      <c r="BL59" s="127"/>
       <c r="BM59" s="62"/>
       <c r="BN59" s="63"/>
       <c r="BO59" s="62"/>
@@ -21826,7 +21846,7 @@
       <c r="BU59" s="63"/>
       <c r="BV59" s="63"/>
       <c r="BW59" s="63"/>
-      <c r="BX59" s="126"/>
+      <c r="BX59" s="127"/>
     </row>
     <row r="60" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E60" s="61"/>
@@ -21849,7 +21869,7 @@
       <c r="Y60" s="93"/>
       <c r="Z60" s="9"/>
       <c r="AB60" s="44"/>
-      <c r="AD60" s="125"/>
+      <c r="AD60" s="126"/>
       <c r="AE60" s="38"/>
       <c r="AF60" s="64"/>
       <c r="AG60" s="38"/>
@@ -21878,79 +21898,79 @@
       <c r="BU60" s="63"/>
       <c r="BV60" s="63"/>
       <c r="BW60" s="63"/>
-      <c r="BX60" s="126"/>
+      <c r="BX60" s="127"/>
     </row>
     <row r="61" s="87" customFormat="true" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="74"/>
       <c r="B61" s="74"/>
       <c r="C61" s="74"/>
       <c r="D61" s="86"/>
-      <c r="E61" s="140"/>
-      <c r="F61" s="140"/>
+      <c r="E61" s="141"/>
+      <c r="F61" s="141"/>
       <c r="G61" s="50"/>
       <c r="H61" s="50"/>
       <c r="I61" s="74"/>
       <c r="J61" s="74"/>
-      <c r="K61" s="141"/>
+      <c r="K61" s="142"/>
       <c r="L61" s="76"/>
       <c r="M61" s="50"/>
-      <c r="N61" s="141"/>
-      <c r="O61" s="141"/>
-      <c r="P61" s="141"/>
-      <c r="Q61" s="140"/>
+      <c r="N61" s="142"/>
+      <c r="O61" s="142"/>
+      <c r="P61" s="142"/>
+      <c r="Q61" s="141"/>
       <c r="R61" s="59"/>
       <c r="S61" s="59"/>
       <c r="T61" s="59"/>
       <c r="V61" s="59"/>
       <c r="W61" s="86"/>
-      <c r="X61" s="142"/>
-      <c r="Y61" s="141"/>
+      <c r="X61" s="143"/>
+      <c r="Y61" s="142"/>
       <c r="Z61" s="86"/>
-      <c r="AA61" s="143"/>
+      <c r="AA61" s="144"/>
       <c r="AB61" s="59"/>
       <c r="AC61" s="77"/>
-      <c r="AD61" s="144"/>
+      <c r="AD61" s="145"/>
       <c r="AE61" s="51"/>
-      <c r="AF61" s="145"/>
+      <c r="AF61" s="146"/>
       <c r="AG61" s="51"/>
-      <c r="AH61" s="145"/>
+      <c r="AH61" s="146"/>
       <c r="AI61" s="51"/>
-      <c r="AK61" s="146"/>
-      <c r="AM61" s="147"/>
-      <c r="AN61" s="147"/>
-      <c r="AR61" s="147"/>
-      <c r="AS61" s="147"/>
-      <c r="AW61" s="147"/>
-      <c r="AX61" s="147"/>
+      <c r="AK61" s="147"/>
+      <c r="AM61" s="148"/>
+      <c r="AN61" s="148"/>
+      <c r="AR61" s="148"/>
+      <c r="AS61" s="148"/>
+      <c r="AW61" s="148"/>
+      <c r="AX61" s="148"/>
       <c r="BA61" s="84"/>
       <c r="BB61" s="84"/>
       <c r="BC61" s="84"/>
       <c r="BD61" s="84"/>
       <c r="BE61" s="79"/>
-      <c r="BF61" s="148"/>
+      <c r="BF61" s="149"/>
       <c r="BG61" s="84"/>
       <c r="BH61" s="84"/>
       <c r="BI61" s="84"/>
       <c r="BJ61" s="84"/>
-      <c r="BK61" s="149"/>
-      <c r="BL61" s="150"/>
+      <c r="BK61" s="150"/>
+      <c r="BL61" s="151"/>
       <c r="BM61" s="84"/>
       <c r="BN61" s="79"/>
       <c r="BO61" s="84"/>
       <c r="BP61" s="74"/>
       <c r="BQ61" s="79"/>
-      <c r="BR61" s="148"/>
+      <c r="BR61" s="149"/>
       <c r="BS61" s="79"/>
       <c r="BT61" s="79"/>
       <c r="BU61" s="79"/>
       <c r="BV61" s="79"/>
       <c r="BW61" s="79"/>
-      <c r="BX61" s="150"/>
+      <c r="BX61" s="151"/>
       <c r="BY61" s="74"/>
-      <c r="CA61" s="147"/>
-      <c r="CB61" s="147"/>
-      <c r="CE61" s="147"/>
-      <c r="CF61" s="147"/>
+      <c r="CA61" s="148"/>
+      <c r="CB61" s="148"/>
+      <c r="CE61" s="148"/>
+      <c r="CF61" s="148"/>
       <c r="CL61" s="74"/>
       <c r="CM61" s="74"/>
       <c r="CN61" s="74"/>
@@ -21978,7 +21998,7 @@
       <c r="Y62" s="93"/>
       <c r="Z62" s="9"/>
       <c r="AB62" s="44"/>
-      <c r="AD62" s="125"/>
+      <c r="AD62" s="126"/>
       <c r="AE62" s="38"/>
       <c r="AF62" s="64"/>
       <c r="AG62" s="38"/>
@@ -22007,7 +22027,7 @@
       <c r="BU62" s="63"/>
       <c r="BV62" s="63"/>
       <c r="BW62" s="63"/>
-      <c r="BX62" s="126"/>
+      <c r="BX62" s="127"/>
     </row>
     <row r="63" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E63" s="61"/>
@@ -22030,7 +22050,7 @@
       <c r="Y63" s="93"/>
       <c r="Z63" s="9"/>
       <c r="AB63" s="44"/>
-      <c r="AD63" s="125"/>
+      <c r="AD63" s="126"/>
       <c r="AE63" s="38"/>
       <c r="AF63" s="64"/>
       <c r="AG63" s="38"/>
@@ -22059,7 +22079,7 @@
       <c r="BU63" s="63"/>
       <c r="BV63" s="63"/>
       <c r="BW63" s="63"/>
-      <c r="BX63" s="126"/>
+      <c r="BX63" s="127"/>
     </row>
     <row r="64" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E64" s="61"/>
@@ -22082,7 +22102,7 @@
       <c r="Y64" s="93"/>
       <c r="Z64" s="9"/>
       <c r="AB64" s="44"/>
-      <c r="AD64" s="125"/>
+      <c r="AD64" s="126"/>
       <c r="AE64" s="38"/>
       <c r="AF64" s="64"/>
       <c r="AG64" s="38"/>
@@ -22100,7 +22120,7 @@
       <c r="BI64" s="62"/>
       <c r="BJ64" s="62"/>
       <c r="BK64" s="65"/>
-      <c r="BL64" s="126"/>
+      <c r="BL64" s="127"/>
       <c r="BM64" s="62"/>
       <c r="BN64" s="63"/>
       <c r="BO64" s="62"/>
@@ -22111,7 +22131,7 @@
       <c r="BU64" s="63"/>
       <c r="BV64" s="63"/>
       <c r="BW64" s="63"/>
-      <c r="BX64" s="126"/>
+      <c r="BX64" s="127"/>
     </row>
     <row r="65" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E65" s="61"/>
@@ -22131,7 +22151,7 @@
       <c r="W65" s="9"/>
       <c r="Y65" s="93"/>
       <c r="Z65" s="9"/>
-      <c r="AD65" s="125"/>
+      <c r="AD65" s="126"/>
       <c r="AE65" s="38"/>
       <c r="AF65" s="64"/>
       <c r="AG65" s="38"/>
@@ -22149,7 +22169,7 @@
       <c r="BI65" s="62"/>
       <c r="BJ65" s="62"/>
       <c r="BK65" s="65"/>
-      <c r="BL65" s="126"/>
+      <c r="BL65" s="127"/>
       <c r="BM65" s="62"/>
       <c r="BN65" s="63"/>
       <c r="BO65" s="62"/>
@@ -22159,7 +22179,7 @@
       <c r="BU65" s="63"/>
       <c r="BV65" s="63"/>
       <c r="BW65" s="63"/>
-      <c r="BX65" s="126"/>
+      <c r="BX65" s="127"/>
     </row>
     <row r="66" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G66" s="37"/>
@@ -22175,7 +22195,7 @@
       <c r="W66" s="9"/>
       <c r="Y66" s="93"/>
       <c r="Z66" s="9"/>
-      <c r="AD66" s="125"/>
+      <c r="AD66" s="126"/>
       <c r="AE66" s="38"/>
       <c r="AF66" s="64"/>
       <c r="AG66" s="38"/>
@@ -22195,19 +22215,19 @@
       <c r="BI66" s="62"/>
       <c r="BJ66" s="63"/>
       <c r="BK66" s="65"/>
-      <c r="BL66" s="126"/>
+      <c r="BL66" s="127"/>
       <c r="BM66" s="62"/>
       <c r="BN66" s="63"/>
       <c r="BO66" s="62"/>
       <c r="BP66" s="10"/>
       <c r="BQ66" s="63"/>
-      <c r="BR66" s="126"/>
+      <c r="BR66" s="127"/>
       <c r="BS66" s="63"/>
       <c r="BT66" s="63"/>
       <c r="BU66" s="63"/>
       <c r="BV66" s="63"/>
       <c r="BW66" s="63"/>
-      <c r="BX66" s="126"/>
+      <c r="BX66" s="127"/>
     </row>
     <row r="67" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G67" s="37"/>
@@ -22222,7 +22242,7 @@
       <c r="W67" s="9"/>
       <c r="Y67" s="93"/>
       <c r="Z67" s="9"/>
-      <c r="AD67" s="125"/>
+      <c r="AD67" s="126"/>
       <c r="AE67" s="38"/>
       <c r="AF67" s="64"/>
       <c r="AG67" s="38"/>
@@ -22245,7 +22265,7 @@
       <c r="T68" s="44"/>
       <c r="W68" s="9"/>
       <c r="Z68" s="9"/>
-      <c r="AD68" s="125"/>
+      <c r="AD68" s="126"/>
       <c r="AE68" s="38"/>
       <c r="AF68" s="64"/>
       <c r="AG68" s="38"/>
@@ -22268,7 +22288,7 @@
       <c r="T69" s="44"/>
       <c r="W69" s="9"/>
       <c r="Z69" s="9"/>
-      <c r="AD69" s="125"/>
+      <c r="AD69" s="126"/>
       <c r="AE69" s="38"/>
       <c r="AF69" s="64"/>
       <c r="AG69" s="38"/>

</xml_diff>